<commit_message>
Implement Pdf writing service
</commit_message>
<xml_diff>
--- a/backend/WimpeyTrack.Api/Templates/template.xlsx
+++ b/backend/WimpeyTrack.Api/Templates/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rossfleming/Projects/wimpey-track/backend/WimpeyTrack.Api/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B06BC3D8-B352-0142-B42A-81E4821E2C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8326FBC8-9467-CC40-B2C1-BFDCA25F3F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="620" windowWidth="25600" windowHeight="26620" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="25600" windowHeight="26620" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Expense Claim Form " sheetId="1" r:id="rId1"/>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="208">
   <si>
     <t>EXPENSES CLAIM FORM  (Use for expenditure incurred from 1 December 2014)</t>
   </si>
@@ -1869,13 +1869,106 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="39" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="8" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="8" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="5" fillId="7" borderId="3" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="39" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="39" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1885,105 +1978,12 @@
     <xf numFmtId="39" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="8" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="8" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="5" fillId="7" borderId="3" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="39" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="39" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2475,78 +2475,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="178" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="178"/>
-      <c r="C1" s="178"/>
-      <c r="D1" s="178"/>
-      <c r="E1" s="178"/>
-      <c r="F1" s="178"/>
-      <c r="G1" s="178"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
-      <c r="J1" s="179"/>
-      <c r="K1" s="179"/>
-      <c r="L1" s="179"/>
-      <c r="M1" s="179"/>
-      <c r="N1" s="179"/>
+      <c r="A1" s="209" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="209"/>
+      <c r="C1" s="209"/>
+      <c r="D1" s="209"/>
+      <c r="E1" s="209"/>
+      <c r="F1" s="209"/>
+      <c r="G1" s="209"/>
+      <c r="H1" s="210"/>
+      <c r="I1" s="210"/>
+      <c r="J1" s="210"/>
+      <c r="K1" s="210"/>
+      <c r="L1" s="210"/>
+      <c r="M1" s="210"/>
+      <c r="N1" s="210"/>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="178"/>
-      <c r="B2" s="178"/>
-      <c r="C2" s="178"/>
-      <c r="D2" s="178"/>
-      <c r="E2" s="178"/>
-      <c r="F2" s="178"/>
-      <c r="G2" s="178"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
-      <c r="J2" s="179"/>
-      <c r="K2" s="179"/>
-      <c r="L2" s="179"/>
-      <c r="M2" s="179"/>
-      <c r="N2" s="179"/>
+      <c r="A2" s="209"/>
+      <c r="B2" s="209"/>
+      <c r="C2" s="209"/>
+      <c r="D2" s="209"/>
+      <c r="E2" s="209"/>
+      <c r="F2" s="209"/>
+      <c r="G2" s="209"/>
+      <c r="H2" s="210"/>
+      <c r="I2" s="210"/>
+      <c r="J2" s="210"/>
+      <c r="K2" s="210"/>
+      <c r="L2" s="210"/>
+      <c r="M2" s="210"/>
+      <c r="N2" s="210"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="178"/>
-      <c r="B3" s="178"/>
-      <c r="C3" s="178"/>
-      <c r="D3" s="178"/>
-      <c r="E3" s="178"/>
-      <c r="F3" s="178"/>
-      <c r="G3" s="178"/>
-      <c r="H3" s="179"/>
-      <c r="I3" s="179"/>
-      <c r="J3" s="179"/>
-      <c r="K3" s="179"/>
-      <c r="L3" s="179"/>
-      <c r="M3" s="179"/>
-      <c r="N3" s="179"/>
+      <c r="A3" s="209"/>
+      <c r="B3" s="209"/>
+      <c r="C3" s="209"/>
+      <c r="D3" s="209"/>
+      <c r="E3" s="209"/>
+      <c r="F3" s="209"/>
+      <c r="G3" s="209"/>
+      <c r="H3" s="210"/>
+      <c r="I3" s="210"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="210"/>
+      <c r="M3" s="210"/>
+      <c r="N3" s="210"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="180" t="s">
+      <c r="A4" s="202" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="180"/>
-      <c r="C4" s="181" t="s">
+      <c r="B4" s="202"/>
+      <c r="C4" s="211" t="s">
         <v>202</v>
       </c>
-      <c r="D4" s="181"/>
-      <c r="E4" s="182" t="s">
+      <c r="D4" s="211"/>
+      <c r="E4" s="212" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="182"/>
-      <c r="G4" s="182"/>
-      <c r="H4" s="182"/>
-      <c r="I4" s="183" t="s">
+      <c r="F4" s="212"/>
+      <c r="G4" s="212"/>
+      <c r="H4" s="212"/>
+      <c r="I4" s="198" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="183"/>
-      <c r="K4" s="183"/>
+      <c r="J4" s="198"/>
+      <c r="K4" s="198"/>
       <c r="L4" s="3" t="s">
         <v>4</v>
       </c>
@@ -2554,25 +2554,25 @@
         <f>'Mileage Detail'!M4</f>
         <v>DIESEL</v>
       </c>
-      <c r="N4" s="182" t="s">
+      <c r="N4" s="212" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="184" t="s">
+      <c r="O4" s="203" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="180"/>
-      <c r="B5" s="180"/>
-      <c r="C5" s="181"/>
-      <c r="D5" s="181"/>
-      <c r="E5" s="182"/>
-      <c r="F5" s="182"/>
-      <c r="G5" s="182"/>
-      <c r="H5" s="182"/>
-      <c r="I5" s="183"/>
-      <c r="J5" s="183"/>
-      <c r="K5" s="183"/>
+      <c r="A5" s="202"/>
+      <c r="B5" s="202"/>
+      <c r="C5" s="211"/>
+      <c r="D5" s="211"/>
+      <c r="E5" s="212"/>
+      <c r="F5" s="212"/>
+      <c r="G5" s="212"/>
+      <c r="H5" s="212"/>
+      <c r="I5" s="198"/>
+      <c r="J5" s="198"/>
+      <c r="K5" s="198"/>
       <c r="L5" s="6" t="s">
         <v>7</v>
       </c>
@@ -2580,133 +2580,133 @@
         <f>'Mileage Detail'!M5</f>
         <v>1600</v>
       </c>
-      <c r="N5" s="182"/>
-      <c r="O5" s="184"/>
+      <c r="N5" s="212"/>
+      <c r="O5" s="203"/>
     </row>
     <row r="6" spans="1:15" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="185" t="s">
+      <c r="A6" s="204" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="185"/>
-      <c r="C6" s="186"/>
-      <c r="D6" s="186"/>
-      <c r="E6" s="186" t="s">
+      <c r="B6" s="204"/>
+      <c r="C6" s="205"/>
+      <c r="D6" s="205"/>
+      <c r="E6" s="205" t="s">
         <v>203</v>
       </c>
-      <c r="F6" s="186"/>
-      <c r="G6" s="186"/>
-      <c r="H6" s="186"/>
-      <c r="I6" s="187"/>
-      <c r="J6" s="187"/>
-      <c r="K6" s="187"/>
-      <c r="L6" s="188" t="s">
+      <c r="F6" s="205"/>
+      <c r="G6" s="205"/>
+      <c r="H6" s="205"/>
+      <c r="I6" s="206"/>
+      <c r="J6" s="206"/>
+      <c r="K6" s="206"/>
+      <c r="L6" s="207" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="184" t="str">
+      <c r="M6" s="203" t="str">
         <f>'Mileage Detail'!M6</f>
         <v>SB65 XCW</v>
       </c>
-      <c r="N6" s="189">
+      <c r="N6" s="208">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
-      </c>
-      <c r="O6" s="184"/>
+        <v>46043</v>
+      </c>
+      <c r="O6" s="203"/>
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="185"/>
-      <c r="B7" s="185"/>
-      <c r="C7" s="186"/>
-      <c r="D7" s="186"/>
-      <c r="E7" s="186"/>
-      <c r="F7" s="186"/>
-      <c r="G7" s="186"/>
-      <c r="H7" s="186"/>
-      <c r="I7" s="187"/>
-      <c r="J7" s="187"/>
-      <c r="K7" s="187"/>
-      <c r="L7" s="188"/>
-      <c r="M7" s="188"/>
-      <c r="N7" s="189"/>
-      <c r="O7" s="184"/>
+      <c r="A7" s="204"/>
+      <c r="B7" s="204"/>
+      <c r="C7" s="205"/>
+      <c r="D7" s="205"/>
+      <c r="E7" s="205"/>
+      <c r="F7" s="205"/>
+      <c r="G7" s="205"/>
+      <c r="H7" s="205"/>
+      <c r="I7" s="206"/>
+      <c r="J7" s="206"/>
+      <c r="K7" s="206"/>
+      <c r="L7" s="207"/>
+      <c r="M7" s="207"/>
+      <c r="N7" s="208"/>
+      <c r="O7" s="203"/>
     </row>
     <row r="8" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="183" t="s">
+      <c r="A8" s="198" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="180" t="s">
+      <c r="B8" s="202" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="183" t="s">
+      <c r="C8" s="198" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="183"/>
-      <c r="E8" s="183" t="s">
+      <c r="D8" s="198"/>
+      <c r="E8" s="198" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="183" t="s">
+      <c r="F8" s="198" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="183" t="s">
+      <c r="G8" s="198" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="183" t="s">
+      <c r="H8" s="198" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="183" t="s">
+      <c r="I8" s="198" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="183" t="s">
+      <c r="J8" s="198" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="183" t="s">
+      <c r="K8" s="198" t="s">
         <v>19</v>
       </c>
-      <c r="L8" s="183" t="s">
+      <c r="L8" s="198" t="s">
         <v>20</v>
       </c>
-      <c r="M8" s="190" t="s">
+      <c r="M8" s="199" t="s">
         <v>21</v>
       </c>
-      <c r="N8" s="183" t="s">
+      <c r="N8" s="198" t="s">
         <v>22</v>
       </c>
-      <c r="O8" s="191" t="s">
+      <c r="O8" s="200" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="183"/>
-      <c r="B9" s="183"/>
-      <c r="C9" s="183"/>
-      <c r="D9" s="183"/>
-      <c r="E9" s="183"/>
-      <c r="F9" s="183"/>
-      <c r="G9" s="183"/>
-      <c r="H9" s="183"/>
-      <c r="I9" s="183"/>
-      <c r="J9" s="183"/>
-      <c r="K9" s="183"/>
-      <c r="L9" s="183"/>
-      <c r="M9" s="190"/>
-      <c r="N9" s="183"/>
-      <c r="O9" s="183"/>
+      <c r="A9" s="198"/>
+      <c r="B9" s="198"/>
+      <c r="C9" s="198"/>
+      <c r="D9" s="198"/>
+      <c r="E9" s="198"/>
+      <c r="F9" s="198"/>
+      <c r="G9" s="198"/>
+      <c r="H9" s="198"/>
+      <c r="I9" s="198"/>
+      <c r="J9" s="198"/>
+      <c r="K9" s="198"/>
+      <c r="L9" s="198"/>
+      <c r="M9" s="199"/>
+      <c r="N9" s="198"/>
+      <c r="O9" s="198"/>
     </row>
     <row r="10" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="183"/>
-      <c r="B10" s="183"/>
-      <c r="C10" s="183"/>
-      <c r="D10" s="183"/>
-      <c r="E10" s="183"/>
-      <c r="F10" s="183"/>
-      <c r="G10" s="183"/>
-      <c r="H10" s="183"/>
-      <c r="I10" s="183"/>
-      <c r="J10" s="183"/>
-      <c r="K10" s="183"/>
-      <c r="L10" s="183"/>
-      <c r="M10" s="190"/>
-      <c r="N10" s="183"/>
-      <c r="O10" s="183"/>
+      <c r="A10" s="198"/>
+      <c r="B10" s="198"/>
+      <c r="C10" s="198"/>
+      <c r="D10" s="198"/>
+      <c r="E10" s="198"/>
+      <c r="F10" s="198"/>
+      <c r="G10" s="198"/>
+      <c r="H10" s="198"/>
+      <c r="I10" s="198"/>
+      <c r="J10" s="198"/>
+      <c r="K10" s="198"/>
+      <c r="L10" s="198"/>
+      <c r="M10" s="199"/>
+      <c r="N10" s="198"/>
+      <c r="O10" s="198"/>
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="8"/>
@@ -3990,10 +3990,10 @@
       <c r="B43" s="42"/>
       <c r="E43" s="42"/>
       <c r="F43" s="42"/>
-      <c r="G43" s="192" t="s">
+      <c r="G43" s="201" t="s">
         <v>34</v>
       </c>
-      <c r="H43" s="192"/>
+      <c r="H43" s="201"/>
       <c r="I43" s="43"/>
       <c r="J43" s="43"/>
       <c r="K43" s="43"/>
@@ -4005,13 +4005,13 @@
       <c r="O43" s="44"/>
     </row>
     <row r="44" spans="1:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B44" s="193">
+      <c r="B44" s="192">
         <f>IF(OR(B49="no",AND(B49="yes",B54=0.25)),0,"WARNING - NON COMPANY CAR USERS WHO HAVE CLAIMED OVER 10,000 BUSINESS MILES IN A TAX YEAR MUST USE A CLAIM PER MILE RATE OF 25p")</f>
         <v>0</v>
       </c>
-      <c r="C44" s="193"/>
-      <c r="D44" s="193"/>
-      <c r="E44" s="193"/>
+      <c r="C44" s="192"/>
+      <c r="D44" s="192"/>
+      <c r="E44" s="192"/>
       <c r="F44" s="42"/>
       <c r="G44" s="45" t="s">
         <v>36</v>
@@ -4037,18 +4037,18 @@
       <c r="N44" s="47">
         <v>95195</v>
       </c>
-      <c r="O44" s="194" t="s">
+      <c r="O44" s="193" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="41"/>
-      <c r="B45" s="193"/>
-      <c r="C45" s="193"/>
-      <c r="D45" s="193"/>
-      <c r="E45" s="193"/>
+      <c r="B45" s="192"/>
+      <c r="C45" s="192"/>
+      <c r="D45" s="192"/>
+      <c r="E45" s="192"/>
       <c r="F45" s="42"/>
-      <c r="G45" s="195">
+      <c r="G45" s="194">
         <f>+G42-H42-SUM(I56,J56,K58,L56,M56,N56)</f>
         <v>0</v>
       </c>
@@ -4067,7 +4067,7 @@
       <c r="N45" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="O45" s="194"/>
+      <c r="O45" s="193"/>
     </row>
     <row r="46" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="41"/>
@@ -4076,7 +4076,7 @@
       <c r="D46" s="50"/>
       <c r="E46" s="50"/>
       <c r="F46" s="42"/>
-      <c r="G46" s="195"/>
+      <c r="G46" s="194"/>
       <c r="H46" s="46"/>
       <c r="I46" s="47"/>
       <c r="J46" s="47"/>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="E47" s="51"/>
       <c r="F47" s="42"/>
-      <c r="G47" s="195"/>
+      <c r="G47" s="194"/>
       <c r="H47" s="46" t="s">
         <v>42</v>
       </c>
@@ -4131,19 +4131,19 @@
       <c r="O48" s="56"/>
     </row>
     <row r="49" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A49" s="196" t="s">
+      <c r="A49" s="184" t="s">
         <v>43</v>
       </c>
-      <c r="B49" s="197" t="s">
+      <c r="B49" s="195" t="s">
         <v>77</v>
       </c>
-      <c r="C49" s="198" t="s">
+      <c r="C49" s="196" t="s">
         <v>45</v>
       </c>
-      <c r="D49" s="198"/>
-      <c r="E49" s="198"/>
-      <c r="F49" s="198"/>
-      <c r="G49" s="199" t="s">
+      <c r="D49" s="196"/>
+      <c r="E49" s="196"/>
+      <c r="F49" s="196"/>
+      <c r="G49" s="197" t="s">
         <v>46</v>
       </c>
       <c r="H49" s="43" t="s">
@@ -4178,13 +4178,13 @@
       </c>
     </row>
     <row r="50" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A50" s="196"/>
-      <c r="B50" s="197"/>
-      <c r="C50" s="198"/>
-      <c r="D50" s="198"/>
-      <c r="E50" s="198"/>
-      <c r="F50" s="198"/>
-      <c r="G50" s="199"/>
+      <c r="A50" s="184"/>
+      <c r="B50" s="195"/>
+      <c r="C50" s="196"/>
+      <c r="D50" s="196"/>
+      <c r="E50" s="196"/>
+      <c r="F50" s="196"/>
+      <c r="G50" s="197"/>
       <c r="H50" s="23"/>
       <c r="I50" s="61"/>
       <c r="J50" s="61"/>
@@ -4195,20 +4195,20 @@
       <c r="O50" s="52"/>
     </row>
     <row r="51" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A51" s="196" t="s">
+      <c r="A51" s="184" t="s">
         <v>48</v>
       </c>
-      <c r="B51" s="204">
+      <c r="B51" s="185">
         <f>'Mileage Detail'!E37</f>
         <v>0</v>
       </c>
-      <c r="C51" s="205" t="s">
+      <c r="C51" s="186" t="s">
         <v>49</v>
       </c>
-      <c r="D51" s="205"/>
-      <c r="E51" s="205"/>
-      <c r="F51" s="205"/>
-      <c r="G51" s="206" t="s">
+      <c r="D51" s="186"/>
+      <c r="E51" s="186"/>
+      <c r="F51" s="186"/>
+      <c r="G51" s="187" t="s">
         <v>50</v>
       </c>
       <c r="H51" s="23" t="s">
@@ -4229,13 +4229,13 @@
       </c>
     </row>
     <row r="52" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A52" s="196"/>
-      <c r="B52" s="196"/>
-      <c r="C52" s="205"/>
-      <c r="D52" s="205"/>
-      <c r="E52" s="205"/>
-      <c r="F52" s="205"/>
-      <c r="G52" s="206"/>
+      <c r="A52" s="184"/>
+      <c r="B52" s="184"/>
+      <c r="C52" s="186"/>
+      <c r="D52" s="186"/>
+      <c r="E52" s="186"/>
+      <c r="F52" s="186"/>
+      <c r="G52" s="187"/>
       <c r="H52" s="23" t="s">
         <v>52</v>
       </c>
@@ -4260,11 +4260,11 @@
       <c r="B53" s="64">
         <v>0.45</v>
       </c>
-      <c r="C53" s="205"/>
-      <c r="D53" s="205"/>
-      <c r="E53" s="205"/>
-      <c r="F53" s="205"/>
-      <c r="G53" s="206"/>
+      <c r="C53" s="186"/>
+      <c r="D53" s="186"/>
+      <c r="E53" s="186"/>
+      <c r="F53" s="186"/>
+      <c r="G53" s="187"/>
       <c r="H53" s="23" t="s">
         <v>54</v>
       </c>
@@ -4295,20 +4295,20 @@
       </c>
     </row>
     <row r="54" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A54" s="207" t="s">
+      <c r="A54" s="188" t="s">
         <v>55</v>
       </c>
-      <c r="B54" s="208">
+      <c r="B54" s="189">
         <f>B51*B53</f>
         <v>0</v>
       </c>
-      <c r="C54" s="209" t="s">
+      <c r="C54" s="190" t="s">
         <v>56</v>
       </c>
-      <c r="D54" s="209"/>
-      <c r="E54" s="209"/>
-      <c r="F54" s="209"/>
-      <c r="G54" s="206"/>
+      <c r="D54" s="190"/>
+      <c r="E54" s="190"/>
+      <c r="F54" s="190"/>
+      <c r="G54" s="187"/>
       <c r="H54" s="23" t="s">
         <v>57</v>
       </c>
@@ -4339,13 +4339,13 @@
       </c>
     </row>
     <row r="55" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A55" s="207"/>
-      <c r="B55" s="207"/>
-      <c r="C55" s="209"/>
-      <c r="D55" s="209"/>
-      <c r="E55" s="209"/>
-      <c r="F55" s="209"/>
-      <c r="G55" s="206"/>
+      <c r="A55" s="188"/>
+      <c r="B55" s="188"/>
+      <c r="C55" s="190"/>
+      <c r="D55" s="190"/>
+      <c r="E55" s="190"/>
+      <c r="F55" s="190"/>
+      <c r="G55" s="187"/>
       <c r="H55" s="23" t="s">
         <v>58</v>
       </c>
@@ -4379,7 +4379,7 @@
       <c r="A56" s="42"/>
       <c r="B56" s="66"/>
       <c r="E56" s="51"/>
-      <c r="G56" s="206"/>
+      <c r="G56" s="187"/>
       <c r="H56" s="23" t="s">
         <v>47</v>
       </c>
@@ -4415,10 +4415,10 @@
     <row r="57" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="68"/>
       <c r="B57" s="69"/>
-      <c r="C57" s="210"/>
-      <c r="D57" s="210"/>
+      <c r="C57" s="191"/>
+      <c r="D57" s="191"/>
       <c r="E57" s="70"/>
-      <c r="G57" s="206"/>
+      <c r="G57" s="187"/>
       <c r="H57" s="71" t="s">
         <v>59</v>
       </c>
@@ -4470,13 +4470,13 @@
       <c r="D59" s="42"/>
     </row>
     <row r="60" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B60" s="212" t="s">
+      <c r="B60" s="180" t="s">
         <v>60</v>
       </c>
-      <c r="C60" s="212"/>
-      <c r="D60" s="212"/>
-      <c r="E60" s="212"/>
-      <c r="F60" s="212"/>
+      <c r="C60" s="180"/>
+      <c r="D60" s="180"/>
+      <c r="E60" s="180"/>
+      <c r="F60" s="180"/>
       <c r="G60" s="80"/>
       <c r="H60" s="81"/>
       <c r="I60" s="81"/>
@@ -4502,10 +4502,10 @@
       <c r="K61" s="88"/>
       <c r="L61" s="88"/>
       <c r="M61" s="88"/>
-      <c r="N61" s="200" t="s">
+      <c r="N61" s="181" t="s">
         <v>62</v>
       </c>
-      <c r="O61" s="200"/>
+      <c r="O61" s="181"/>
     </row>
     <row r="62" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62" s="89"/>
@@ -4520,8 +4520,8 @@
       <c r="K62" s="88"/>
       <c r="L62" s="88"/>
       <c r="M62" s="92"/>
-      <c r="N62" s="200"/>
-      <c r="O62" s="200"/>
+      <c r="N62" s="181"/>
+      <c r="O62" s="181"/>
     </row>
     <row r="63" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B63" s="89"/>
@@ -4529,21 +4529,21 @@
         <v>63</v>
       </c>
       <c r="D63" s="93"/>
-      <c r="E63" s="201"/>
-      <c r="F63" s="201"/>
+      <c r="E63" s="182"/>
+      <c r="F63" s="182"/>
       <c r="G63" s="91"/>
       <c r="H63" s="94" t="s">
         <v>64</v>
       </c>
-      <c r="I63" s="202"/>
-      <c r="J63" s="202"/>
-      <c r="K63" s="202"/>
+      <c r="I63" s="183"/>
+      <c r="J63" s="183"/>
+      <c r="K63" s="183"/>
       <c r="L63" s="96" t="s">
         <v>11</v>
       </c>
       <c r="M63" s="95"/>
-      <c r="N63" s="200"/>
-      <c r="O63" s="200"/>
+      <c r="N63" s="181"/>
+      <c r="O63" s="181"/>
     </row>
     <row r="64" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B64" s="89"/>
@@ -4733,10 +4733,10 @@
       <c r="E74" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F74" s="203" t="s">
+      <c r="F74" s="178" t="s">
         <v>76</v>
       </c>
-      <c r="G74" s="203"/>
+      <c r="G74" s="178"/>
       <c r="H74" s="116"/>
       <c r="I74" s="114"/>
       <c r="J74" s="70"/>
@@ -4759,10 +4759,10 @@
       <c r="E75" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F75" s="203" t="s">
+      <c r="F75" s="178" t="s">
         <v>80</v>
       </c>
-      <c r="G75" s="203"/>
+      <c r="G75" s="178"/>
       <c r="H75" s="5"/>
       <c r="I75" s="114"/>
       <c r="J75" s="70"/>
@@ -4783,10 +4783,10 @@
       <c r="E76" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F76" s="203" t="s">
+      <c r="F76" s="178" t="s">
         <v>83</v>
       </c>
-      <c r="G76" s="203"/>
+      <c r="G76" s="178"/>
       <c r="H76" s="5"/>
       <c r="I76" s="114"/>
       <c r="J76" s="70"/>
@@ -4807,10 +4807,10 @@
       <c r="E77" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F77" s="211" t="s">
+      <c r="F77" s="179" t="s">
         <v>86</v>
       </c>
-      <c r="G77" s="211"/>
+      <c r="G77" s="179"/>
       <c r="H77" s="114"/>
       <c r="I77" s="114"/>
       <c r="J77" s="70"/>
@@ -4834,10 +4834,10 @@
       <c r="E78" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F78" s="203" t="s">
+      <c r="F78" s="178" t="s">
         <v>89</v>
       </c>
-      <c r="G78" s="203"/>
+      <c r="G78" s="178"/>
       <c r="H78" s="114"/>
       <c r="I78" s="114"/>
       <c r="J78" s="70"/>
@@ -4932,11 +4932,43 @@
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="F77:G77"/>
-    <mergeCell ref="F78:G78"/>
-    <mergeCell ref="B60:F60"/>
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="H1:N3"/>
+    <mergeCell ref="A4:B5"/>
+    <mergeCell ref="C4:D5"/>
+    <mergeCell ref="E4:H5"/>
+    <mergeCell ref="I4:K5"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O7"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="C6:D7"/>
+    <mergeCell ref="E6:H7"/>
+    <mergeCell ref="I6:K7"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="N8:N10"/>
+    <mergeCell ref="O8:O10"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="B44:E45"/>
+    <mergeCell ref="O44:O45"/>
+    <mergeCell ref="G45:G47"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:F50"/>
+    <mergeCell ref="G49:G50"/>
     <mergeCell ref="N61:O63"/>
     <mergeCell ref="E63:F63"/>
     <mergeCell ref="I63:K63"/>
@@ -4949,43 +4981,11 @@
     <mergeCell ref="B54:B55"/>
     <mergeCell ref="C54:F55"/>
     <mergeCell ref="C57:D57"/>
-    <mergeCell ref="B44:E45"/>
-    <mergeCell ref="O44:O45"/>
-    <mergeCell ref="G45:G47"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:F50"/>
-    <mergeCell ref="G49:G50"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="N8:N10"/>
-    <mergeCell ref="O8:O10"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G8:G10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="O4:O7"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="C6:D7"/>
-    <mergeCell ref="E6:H7"/>
-    <mergeCell ref="I6:K7"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="A1:G3"/>
-    <mergeCell ref="H1:N3"/>
-    <mergeCell ref="A4:B5"/>
-    <mergeCell ref="C4:D5"/>
-    <mergeCell ref="E4:H5"/>
-    <mergeCell ref="I4:K5"/>
-    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="B60:F60"/>
   </mergeCells>
   <conditionalFormatting sqref="B44">
     <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Warning">
@@ -5048,79 +5048,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="178" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="178"/>
-      <c r="C1" s="178"/>
-      <c r="D1" s="178"/>
-      <c r="E1" s="178"/>
-      <c r="F1" s="178"/>
-      <c r="G1" s="178"/>
-      <c r="H1" s="179"/>
-      <c r="I1" s="179"/>
-      <c r="J1" s="179"/>
-      <c r="K1" s="179"/>
-      <c r="L1" s="179"/>
-      <c r="M1" s="179"/>
-      <c r="N1" s="179"/>
+      <c r="A1" s="209" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="209"/>
+      <c r="C1" s="209"/>
+      <c r="D1" s="209"/>
+      <c r="E1" s="209"/>
+      <c r="F1" s="209"/>
+      <c r="G1" s="209"/>
+      <c r="H1" s="210"/>
+      <c r="I1" s="210"/>
+      <c r="J1" s="210"/>
+      <c r="K1" s="210"/>
+      <c r="L1" s="210"/>
+      <c r="M1" s="210"/>
+      <c r="N1" s="210"/>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="178"/>
-      <c r="B2" s="178"/>
-      <c r="C2" s="178"/>
-      <c r="D2" s="178"/>
-      <c r="E2" s="178"/>
-      <c r="F2" s="178"/>
-      <c r="G2" s="178"/>
-      <c r="H2" s="179"/>
-      <c r="I2" s="179"/>
-      <c r="J2" s="179"/>
-      <c r="K2" s="179"/>
-      <c r="L2" s="179"/>
-      <c r="M2" s="179"/>
-      <c r="N2" s="179"/>
+      <c r="A2" s="209"/>
+      <c r="B2" s="209"/>
+      <c r="C2" s="209"/>
+      <c r="D2" s="209"/>
+      <c r="E2" s="209"/>
+      <c r="F2" s="209"/>
+      <c r="G2" s="209"/>
+      <c r="H2" s="210"/>
+      <c r="I2" s="210"/>
+      <c r="J2" s="210"/>
+      <c r="K2" s="210"/>
+      <c r="L2" s="210"/>
+      <c r="M2" s="210"/>
+      <c r="N2" s="210"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="178"/>
-      <c r="B3" s="178"/>
-      <c r="C3" s="178"/>
-      <c r="D3" s="178"/>
-      <c r="E3" s="178"/>
-      <c r="F3" s="178"/>
-      <c r="G3" s="178"/>
-      <c r="H3" s="179"/>
-      <c r="I3" s="179"/>
-      <c r="J3" s="179"/>
-      <c r="K3" s="179"/>
-      <c r="L3" s="179"/>
-      <c r="M3" s="179"/>
-      <c r="N3" s="179"/>
+      <c r="A3" s="209"/>
+      <c r="B3" s="209"/>
+      <c r="C3" s="209"/>
+      <c r="D3" s="209"/>
+      <c r="E3" s="209"/>
+      <c r="F3" s="209"/>
+      <c r="G3" s="209"/>
+      <c r="H3" s="210"/>
+      <c r="I3" s="210"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="210"/>
+      <c r="M3" s="210"/>
+      <c r="N3" s="210"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="180" t="s">
+      <c r="A4" s="202" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="180"/>
-      <c r="C4" s="213" t="str">
+      <c r="B4" s="202"/>
+      <c r="C4" s="216" t="str">
         <f>'Expense Claim Form '!C4:D5</f>
         <v>Brian Fleming</v>
       </c>
-      <c r="D4" s="213"/>
-      <c r="E4" s="182" t="s">
+      <c r="D4" s="216"/>
+      <c r="E4" s="212" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="182"/>
-      <c r="G4" s="182"/>
-      <c r="H4" s="182"/>
-      <c r="I4" s="183" t="s">
+      <c r="F4" s="212"/>
+      <c r="G4" s="212"/>
+      <c r="H4" s="212"/>
+      <c r="I4" s="198" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="183"/>
-      <c r="K4" s="183"/>
+      <c r="J4" s="198"/>
+      <c r="K4" s="198"/>
       <c r="L4" s="3" t="s">
         <v>4</v>
       </c>
@@ -5128,25 +5128,25 @@
         <f>'Mileage Detail'!M4</f>
         <v>DIESEL</v>
       </c>
-      <c r="N4" s="182" t="s">
+      <c r="N4" s="212" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="184" t="s">
+      <c r="O4" s="203" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="180"/>
-      <c r="B5" s="180"/>
-      <c r="C5" s="213"/>
-      <c r="D5" s="213"/>
-      <c r="E5" s="182"/>
-      <c r="F5" s="182"/>
-      <c r="G5" s="182"/>
-      <c r="H5" s="182"/>
-      <c r="I5" s="183"/>
-      <c r="J5" s="183"/>
-      <c r="K5" s="183"/>
+      <c r="A5" s="202"/>
+      <c r="B5" s="202"/>
+      <c r="C5" s="216"/>
+      <c r="D5" s="216"/>
+      <c r="E5" s="212"/>
+      <c r="F5" s="212"/>
+      <c r="G5" s="212"/>
+      <c r="H5" s="212"/>
+      <c r="I5" s="198"/>
+      <c r="J5" s="198"/>
+      <c r="K5" s="198"/>
       <c r="L5" s="6" t="s">
         <v>7</v>
       </c>
@@ -5154,140 +5154,140 @@
         <f>'Mileage Detail'!M5</f>
         <v>1600</v>
       </c>
-      <c r="N5" s="182"/>
-      <c r="O5" s="184"/>
+      <c r="N5" s="212"/>
+      <c r="O5" s="203"/>
     </row>
     <row r="6" spans="1:15" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="185" t="s">
+      <c r="A6" s="204" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="185"/>
-      <c r="C6" s="213">
+      <c r="B6" s="204"/>
+      <c r="C6" s="216">
         <f>'Expense Claim Form '!C6:D7</f>
         <v>0</v>
       </c>
-      <c r="D6" s="213"/>
-      <c r="E6" s="213" t="str">
+      <c r="D6" s="216"/>
+      <c r="E6" s="216" t="str">
         <f>'Expense Claim Form '!E6:H7</f>
         <v>Taylor Wimpey West of Scotland</v>
       </c>
-      <c r="F6" s="213"/>
-      <c r="G6" s="213"/>
-      <c r="H6" s="213"/>
-      <c r="I6" s="184">
+      <c r="F6" s="216"/>
+      <c r="G6" s="216"/>
+      <c r="H6" s="216"/>
+      <c r="I6" s="203">
         <f>'Expense Claim Form '!I6:K7</f>
         <v>0</v>
       </c>
-      <c r="J6" s="184"/>
-      <c r="K6" s="184"/>
-      <c r="L6" s="188" t="s">
+      <c r="J6" s="203"/>
+      <c r="K6" s="203"/>
+      <c r="L6" s="207" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="184" t="str">
+      <c r="M6" s="203" t="str">
         <f>'Mileage Detail'!M6</f>
         <v>SB65 XCW</v>
       </c>
-      <c r="N6" s="189">
+      <c r="N6" s="208">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
-      </c>
-      <c r="O6" s="184"/>
+        <v>46043</v>
+      </c>
+      <c r="O6" s="203"/>
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="185"/>
-      <c r="B7" s="185"/>
-      <c r="C7" s="213"/>
-      <c r="D7" s="213"/>
-      <c r="E7" s="213"/>
-      <c r="F7" s="213"/>
-      <c r="G7" s="213"/>
-      <c r="H7" s="213"/>
-      <c r="I7" s="184"/>
-      <c r="J7" s="184"/>
-      <c r="K7" s="184"/>
-      <c r="L7" s="188"/>
-      <c r="M7" s="188"/>
-      <c r="N7" s="189"/>
-      <c r="O7" s="184"/>
+      <c r="A7" s="204"/>
+      <c r="B7" s="204"/>
+      <c r="C7" s="216"/>
+      <c r="D7" s="216"/>
+      <c r="E7" s="216"/>
+      <c r="F7" s="216"/>
+      <c r="G7" s="216"/>
+      <c r="H7" s="216"/>
+      <c r="I7" s="203"/>
+      <c r="J7" s="203"/>
+      <c r="K7" s="203"/>
+      <c r="L7" s="207"/>
+      <c r="M7" s="207"/>
+      <c r="N7" s="208"/>
+      <c r="O7" s="203"/>
     </row>
     <row r="8" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="183" t="s">
+      <c r="A8" s="198" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="180" t="s">
+      <c r="B8" s="202" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="183" t="s">
+      <c r="C8" s="198" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="183"/>
-      <c r="E8" s="183" t="s">
+      <c r="D8" s="198"/>
+      <c r="E8" s="198" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="183" t="s">
+      <c r="F8" s="198" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="183" t="s">
+      <c r="G8" s="198" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="183" t="s">
+      <c r="H8" s="198" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="183" t="s">
+      <c r="I8" s="198" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="183" t="s">
+      <c r="J8" s="198" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="183" t="s">
+      <c r="K8" s="198" t="s">
         <v>19</v>
       </c>
-      <c r="L8" s="183" t="s">
+      <c r="L8" s="198" t="s">
         <v>20</v>
       </c>
-      <c r="M8" s="190" t="s">
+      <c r="M8" s="199" t="s">
         <v>21</v>
       </c>
-      <c r="N8" s="183" t="s">
+      <c r="N8" s="198" t="s">
         <v>22</v>
       </c>
-      <c r="O8" s="191" t="s">
+      <c r="O8" s="200" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="183"/>
-      <c r="B9" s="183"/>
-      <c r="C9" s="183"/>
-      <c r="D9" s="183"/>
-      <c r="E9" s="183"/>
-      <c r="F9" s="183"/>
-      <c r="G9" s="183"/>
-      <c r="H9" s="183"/>
-      <c r="I9" s="183"/>
-      <c r="J9" s="183"/>
-      <c r="K9" s="183"/>
-      <c r="L9" s="183"/>
-      <c r="M9" s="190"/>
-      <c r="N9" s="183"/>
-      <c r="O9" s="183"/>
+      <c r="A9" s="198"/>
+      <c r="B9" s="198"/>
+      <c r="C9" s="198"/>
+      <c r="D9" s="198"/>
+      <c r="E9" s="198"/>
+      <c r="F9" s="198"/>
+      <c r="G9" s="198"/>
+      <c r="H9" s="198"/>
+      <c r="I9" s="198"/>
+      <c r="J9" s="198"/>
+      <c r="K9" s="198"/>
+      <c r="L9" s="198"/>
+      <c r="M9" s="199"/>
+      <c r="N9" s="198"/>
+      <c r="O9" s="198"/>
     </row>
     <row r="10" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="183"/>
-      <c r="B10" s="183"/>
-      <c r="C10" s="183"/>
-      <c r="D10" s="183"/>
-      <c r="E10" s="183"/>
-      <c r="F10" s="183"/>
-      <c r="G10" s="183"/>
-      <c r="H10" s="183"/>
-      <c r="I10" s="183"/>
-      <c r="J10" s="183"/>
-      <c r="K10" s="183"/>
-      <c r="L10" s="183"/>
-      <c r="M10" s="190"/>
-      <c r="N10" s="183"/>
-      <c r="O10" s="183"/>
+      <c r="A10" s="198"/>
+      <c r="B10" s="198"/>
+      <c r="C10" s="198"/>
+      <c r="D10" s="198"/>
+      <c r="E10" s="198"/>
+      <c r="F10" s="198"/>
+      <c r="G10" s="198"/>
+      <c r="H10" s="198"/>
+      <c r="I10" s="198"/>
+      <c r="J10" s="198"/>
+      <c r="K10" s="198"/>
+      <c r="L10" s="198"/>
+      <c r="M10" s="199"/>
+      <c r="N10" s="198"/>
+      <c r="O10" s="198"/>
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="8"/>
@@ -6918,10 +6918,10 @@
       <c r="B53" s="42"/>
       <c r="E53" s="42"/>
       <c r="F53" s="42"/>
-      <c r="G53" s="192" t="s">
+      <c r="G53" s="201" t="s">
         <v>34</v>
       </c>
-      <c r="H53" s="192"/>
+      <c r="H53" s="201"/>
       <c r="I53" s="43"/>
       <c r="J53" s="43"/>
       <c r="K53" s="43"/>
@@ -6933,10 +6933,10 @@
       <c r="O53" s="44"/>
     </row>
     <row r="54" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B54" s="214"/>
-      <c r="C54" s="214"/>
-      <c r="D54" s="214"/>
-      <c r="E54" s="214"/>
+      <c r="B54" s="213"/>
+      <c r="C54" s="213"/>
+      <c r="D54" s="213"/>
+      <c r="E54" s="213"/>
       <c r="G54" s="45" t="s">
         <v>36</v>
       </c>
@@ -6961,16 +6961,16 @@
       <c r="N54" s="47">
         <v>95195</v>
       </c>
-      <c r="O54" s="194" t="s">
+      <c r="O54" s="193" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="55" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B55" s="214"/>
-      <c r="C55" s="214"/>
-      <c r="D55" s="214"/>
-      <c r="E55" s="214"/>
-      <c r="G55" s="195">
+      <c r="B55" s="213"/>
+      <c r="C55" s="213"/>
+      <c r="D55" s="213"/>
+      <c r="E55" s="213"/>
+      <c r="G55" s="194">
         <f>+G52-H52-SUM(I66:N66)</f>
         <v>0</v>
       </c>
@@ -6989,7 +6989,7 @@
       <c r="N55" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="O55" s="194"/>
+      <c r="O55" s="193"/>
     </row>
     <row r="56" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="41"/>
@@ -6998,7 +6998,7 @@
       <c r="D56" s="50"/>
       <c r="E56" s="50"/>
       <c r="F56" s="42"/>
-      <c r="G56" s="195"/>
+      <c r="G56" s="194"/>
       <c r="H56" s="46"/>
       <c r="I56" s="47"/>
       <c r="J56" s="47"/>
@@ -7009,7 +7009,7 @@
       <c r="O56" s="48"/>
     </row>
     <row r="57" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G57" s="195"/>
+      <c r="G57" s="194"/>
       <c r="H57" s="46" t="s">
         <v>42</v>
       </c>
@@ -7045,13 +7045,13 @@
       <c r="O58" s="56"/>
     </row>
     <row r="59" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A59" s="214"/>
-      <c r="B59" s="214"/>
-      <c r="C59" s="214"/>
-      <c r="D59" s="214"/>
-      <c r="E59" s="214"/>
-      <c r="F59" s="214"/>
-      <c r="G59" s="199" t="s">
+      <c r="A59" s="213"/>
+      <c r="B59" s="213"/>
+      <c r="C59" s="213"/>
+      <c r="D59" s="213"/>
+      <c r="E59" s="213"/>
+      <c r="F59" s="213"/>
+      <c r="G59" s="197" t="s">
         <v>46</v>
       </c>
       <c r="H59" s="43" t="s">
@@ -7086,13 +7086,13 @@
       </c>
     </row>
     <row r="60" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A60" s="214"/>
-      <c r="B60" s="214"/>
-      <c r="C60" s="214"/>
-      <c r="D60" s="214"/>
-      <c r="E60" s="214"/>
-      <c r="F60" s="214"/>
-      <c r="G60" s="199"/>
+      <c r="A60" s="213"/>
+      <c r="B60" s="213"/>
+      <c r="C60" s="213"/>
+      <c r="D60" s="213"/>
+      <c r="E60" s="213"/>
+      <c r="F60" s="213"/>
+      <c r="G60" s="197"/>
       <c r="H60" s="23"/>
       <c r="I60" s="21"/>
       <c r="J60" s="21"/>
@@ -7103,13 +7103,13 @@
       <c r="O60" s="52"/>
     </row>
     <row r="61" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A61" s="214"/>
-      <c r="B61" s="215"/>
-      <c r="C61" s="214"/>
-      <c r="D61" s="214"/>
-      <c r="E61" s="214"/>
-      <c r="F61" s="214"/>
-      <c r="G61" s="216" t="s">
+      <c r="A61" s="213"/>
+      <c r="B61" s="214"/>
+      <c r="C61" s="213"/>
+      <c r="D61" s="213"/>
+      <c r="E61" s="213"/>
+      <c r="F61" s="213"/>
+      <c r="G61" s="215" t="s">
         <v>50</v>
       </c>
       <c r="H61" s="23" t="s">
@@ -7130,13 +7130,13 @@
       </c>
     </row>
     <row r="62" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A62" s="214"/>
-      <c r="B62" s="214"/>
-      <c r="C62" s="214"/>
-      <c r="D62" s="214"/>
-      <c r="E62" s="214"/>
-      <c r="F62" s="214"/>
-      <c r="G62" s="216"/>
+      <c r="A62" s="213"/>
+      <c r="B62" s="213"/>
+      <c r="C62" s="213"/>
+      <c r="D62" s="213"/>
+      <c r="E62" s="213"/>
+      <c r="F62" s="213"/>
+      <c r="G62" s="215"/>
       <c r="H62" s="23" t="s">
         <v>52</v>
       </c>
@@ -7156,11 +7156,11 @@
     </row>
     <row r="63" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B63"/>
-      <c r="C63" s="214"/>
-      <c r="D63" s="214"/>
-      <c r="E63" s="214"/>
-      <c r="F63" s="214"/>
-      <c r="G63" s="216"/>
+      <c r="C63" s="213"/>
+      <c r="D63" s="213"/>
+      <c r="E63" s="213"/>
+      <c r="F63" s="213"/>
+      <c r="G63" s="215"/>
       <c r="H63" s="23" t="s">
         <v>54</v>
       </c>
@@ -7191,13 +7191,13 @@
       </c>
     </row>
     <row r="64" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A64" s="214"/>
-      <c r="B64" s="215"/>
-      <c r="C64" s="214"/>
-      <c r="D64" s="214"/>
-      <c r="E64" s="214"/>
-      <c r="F64" s="214"/>
-      <c r="G64" s="216"/>
+      <c r="A64" s="213"/>
+      <c r="B64" s="214"/>
+      <c r="C64" s="213"/>
+      <c r="D64" s="213"/>
+      <c r="E64" s="213"/>
+      <c r="F64" s="213"/>
+      <c r="G64" s="215"/>
       <c r="H64" s="23" t="s">
         <v>57</v>
       </c>
@@ -7228,13 +7228,13 @@
       </c>
     </row>
     <row r="65" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A65" s="214"/>
-      <c r="B65" s="214"/>
-      <c r="C65" s="214"/>
-      <c r="D65" s="214"/>
-      <c r="E65" s="214"/>
-      <c r="F65" s="214"/>
-      <c r="G65" s="216"/>
+      <c r="A65" s="213"/>
+      <c r="B65" s="213"/>
+      <c r="C65" s="213"/>
+      <c r="D65" s="213"/>
+      <c r="E65" s="213"/>
+      <c r="F65" s="213"/>
+      <c r="G65" s="215"/>
       <c r="H65" s="23" t="s">
         <v>58</v>
       </c>
@@ -7265,7 +7265,7 @@
       </c>
     </row>
     <row r="66" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G66" s="216"/>
+      <c r="G66" s="215"/>
       <c r="H66" s="23" t="s">
         <v>47</v>
       </c>
@@ -7300,9 +7300,9 @@
     </row>
     <row r="67" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B67"/>
-      <c r="C67" s="214"/>
-      <c r="D67" s="214"/>
-      <c r="G67" s="216"/>
+      <c r="C67" s="213"/>
+      <c r="D67" s="213"/>
+      <c r="G67" s="215"/>
       <c r="H67" s="54" t="s">
         <v>59</v>
       </c>
@@ -7403,10 +7403,10 @@
       <c r="E72" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F72" s="203" t="s">
+      <c r="F72" s="178" t="s">
         <v>76</v>
       </c>
-      <c r="G72" s="203"/>
+      <c r="G72" s="178"/>
       <c r="H72" s="116"/>
       <c r="I72" s="114"/>
       <c r="J72" s="70"/>
@@ -7429,10 +7429,10 @@
       <c r="E73" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F73" s="203" t="s">
+      <c r="F73" s="178" t="s">
         <v>80</v>
       </c>
-      <c r="G73" s="203"/>
+      <c r="G73" s="178"/>
       <c r="H73" s="5"/>
       <c r="I73" s="114"/>
       <c r="J73" s="70"/>
@@ -7453,10 +7453,10 @@
       <c r="E74" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F74" s="203" t="s">
+      <c r="F74" s="178" t="s">
         <v>83</v>
       </c>
-      <c r="G74" s="203"/>
+      <c r="G74" s="178"/>
       <c r="H74" s="5"/>
       <c r="I74" s="114"/>
       <c r="J74" s="70"/>
@@ -7477,10 +7477,10 @@
       <c r="E75" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F75" s="211" t="s">
+      <c r="F75" s="179" t="s">
         <v>86</v>
       </c>
-      <c r="G75" s="211"/>
+      <c r="G75" s="179"/>
       <c r="H75" s="114"/>
       <c r="I75" s="114"/>
       <c r="J75" s="70"/>
@@ -7504,10 +7504,10 @@
       <c r="E76" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F76" s="203" t="s">
+      <c r="F76" s="178" t="s">
         <v>89</v>
       </c>
-      <c r="G76" s="203"/>
+      <c r="G76" s="178"/>
       <c r="H76" s="114"/>
       <c r="I76" s="114"/>
       <c r="J76" s="70"/>
@@ -7565,26 +7565,26 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="F73:G73"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="A61:A62"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="C61:F63"/>
-    <mergeCell ref="G61:G67"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:F65"/>
-    <mergeCell ref="C67:D67"/>
-    <mergeCell ref="B54:E55"/>
-    <mergeCell ref="O54:O55"/>
-    <mergeCell ref="G55:G57"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:F60"/>
-    <mergeCell ref="G59:G60"/>
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="H1:N3"/>
+    <mergeCell ref="A4:B5"/>
+    <mergeCell ref="C4:D5"/>
+    <mergeCell ref="E4:H5"/>
+    <mergeCell ref="I4:K5"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O7"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="C6:D7"/>
+    <mergeCell ref="E6:H7"/>
+    <mergeCell ref="I6:K7"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="F8:F10"/>
     <mergeCell ref="L8:L10"/>
     <mergeCell ref="M8:M10"/>
     <mergeCell ref="N8:N10"/>
@@ -7595,26 +7595,26 @@
     <mergeCell ref="I8:I10"/>
     <mergeCell ref="J8:J10"/>
     <mergeCell ref="K8:K10"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="O4:O7"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="C6:D7"/>
-    <mergeCell ref="E6:H7"/>
-    <mergeCell ref="I6:K7"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="A1:G3"/>
-    <mergeCell ref="H1:N3"/>
-    <mergeCell ref="A4:B5"/>
-    <mergeCell ref="C4:D5"/>
-    <mergeCell ref="E4:H5"/>
-    <mergeCell ref="I4:K5"/>
-    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="B54:E55"/>
+    <mergeCell ref="O54:O55"/>
+    <mergeCell ref="G55:G57"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:F60"/>
+    <mergeCell ref="G59:G60"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="C61:F63"/>
+    <mergeCell ref="G61:G67"/>
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:F65"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="F76:G76"/>
   </mergeCells>
   <conditionalFormatting sqref="B54">
     <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Warning">
@@ -10560,7 +10560,9 @@
       <c r="L4" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="131"/>
+      <c r="M4" s="131" t="s">
+        <v>204</v>
+      </c>
       <c r="N4" s="70"/>
       <c r="O4" s="70"/>
       <c r="P4" s="70"/>
@@ -10585,7 +10587,9 @@
       <c r="L5" s="134" t="s">
         <v>7</v>
       </c>
-      <c r="M5" s="131"/>
+      <c r="M5" s="131">
+        <v>1600</v>
+      </c>
       <c r="N5" s="70"/>
       <c r="O5" s="70"/>
       <c r="P5" s="70"/>
@@ -10617,7 +10621,9 @@
       <c r="L6" s="144" t="s">
         <v>106</v>
       </c>
-      <c r="M6" s="131"/>
+      <c r="M6" s="131" t="s">
+        <v>205</v>
+      </c>
       <c r="N6" s="70"/>
       <c r="O6" s="70"/>
       <c r="P6" s="70"/>
@@ -10649,7 +10655,9 @@
       <c r="L7" s="144" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="131"/>
+      <c r="M7" s="131" t="s">
+        <v>206</v>
+      </c>
       <c r="N7" s="70"/>
       <c r="O7" s="70"/>
       <c r="P7" s="70"/>

</xml_diff>

<commit_message>
Add profile data to expense sheets
</commit_message>
<xml_diff>
--- a/backend/WimpeyTrack.Api/Templates/template.xlsx
+++ b/backend/WimpeyTrack.Api/Templates/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rossfleming/Projects/wimpey-track/backend/WimpeyTrack.Api/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8326FBC8-9467-CC40-B2C1-BFDCA25F3F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC248F8-0BFA-2B48-B962-253250013BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="25600" windowHeight="26620" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25600" yWindow="620" windowWidth="25600" windowHeight="26620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Expense Claim Form " sheetId="1" r:id="rId1"/>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="203">
   <si>
     <t>EXPENSES CLAIM FORM  (Use for expenditure incurred from 1 December 2014)</t>
   </si>
@@ -706,21 +706,6 @@
   </si>
   <si>
     <t>In order to claim the passenger mileage rate the employee must have a genuine business reason for having a passenger (eg attending a training course away from their normal place of work, where the payment of the passenger mileage rate represents a cost-saving to the Business Unit).  The passenger mileage rate is not payable in respect of an employee's commute to their normal place of work.  The passsenger must be a TW employee and not a contractor/business contact.</t>
-  </si>
-  <si>
-    <t>Brian Fleming</t>
-  </si>
-  <si>
-    <t>Taylor Wimpey West of Scotland</t>
-  </si>
-  <si>
-    <t>DIESEL</t>
-  </si>
-  <si>
-    <t>SB65 XCW</t>
-  </si>
-  <si>
-    <t>CITREON</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -1869,56 +1854,65 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="39" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="39" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="8" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="39" fontId="8" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="39" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="5" fillId="7" borderId="3" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="39" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1930,60 +1924,51 @@
     <xf numFmtId="39" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="39" fontId="8" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="8" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="39" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="39" fontId="5" fillId="7" borderId="3" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="39" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="39" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="39" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="39" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2475,238 +2460,234 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="209" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="209"/>
-      <c r="C1" s="209"/>
-      <c r="D1" s="209"/>
-      <c r="E1" s="209"/>
-      <c r="F1" s="209"/>
-      <c r="G1" s="209"/>
-      <c r="H1" s="210"/>
-      <c r="I1" s="210"/>
-      <c r="J1" s="210"/>
-      <c r="K1" s="210"/>
-      <c r="L1" s="210"/>
-      <c r="M1" s="210"/>
-      <c r="N1" s="210"/>
+      <c r="A1" s="178" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="179"/>
+      <c r="I1" s="179"/>
+      <c r="J1" s="179"/>
+      <c r="K1" s="179"/>
+      <c r="L1" s="179"/>
+      <c r="M1" s="179"/>
+      <c r="N1" s="179"/>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="209"/>
-      <c r="B2" s="209"/>
-      <c r="C2" s="209"/>
-      <c r="D2" s="209"/>
-      <c r="E2" s="209"/>
-      <c r="F2" s="209"/>
-      <c r="G2" s="209"/>
-      <c r="H2" s="210"/>
-      <c r="I2" s="210"/>
-      <c r="J2" s="210"/>
-      <c r="K2" s="210"/>
-      <c r="L2" s="210"/>
-      <c r="M2" s="210"/>
-      <c r="N2" s="210"/>
+      <c r="A2" s="178"/>
+      <c r="B2" s="178"/>
+      <c r="C2" s="178"/>
+      <c r="D2" s="178"/>
+      <c r="E2" s="178"/>
+      <c r="F2" s="178"/>
+      <c r="G2" s="178"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
+      <c r="L2" s="179"/>
+      <c r="M2" s="179"/>
+      <c r="N2" s="179"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="209"/>
-      <c r="B3" s="209"/>
-      <c r="C3" s="209"/>
-      <c r="D3" s="209"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="209"/>
-      <c r="G3" s="209"/>
-      <c r="H3" s="210"/>
-      <c r="I3" s="210"/>
-      <c r="J3" s="210"/>
-      <c r="K3" s="210"/>
-      <c r="L3" s="210"/>
-      <c r="M3" s="210"/>
-      <c r="N3" s="210"/>
+      <c r="A3" s="178"/>
+      <c r="B3" s="178"/>
+      <c r="C3" s="178"/>
+      <c r="D3" s="178"/>
+      <c r="E3" s="178"/>
+      <c r="F3" s="178"/>
+      <c r="G3" s="178"/>
+      <c r="H3" s="179"/>
+      <c r="I3" s="179"/>
+      <c r="J3" s="179"/>
+      <c r="K3" s="179"/>
+      <c r="L3" s="179"/>
+      <c r="M3" s="179"/>
+      <c r="N3" s="179"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="202" t="s">
+      <c r="A4" s="180" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="202"/>
-      <c r="C4" s="211" t="s">
-        <v>202</v>
-      </c>
-      <c r="D4" s="211"/>
-      <c r="E4" s="212" t="s">
+      <c r="B4" s="180"/>
+      <c r="C4" s="181"/>
+      <c r="D4" s="181"/>
+      <c r="E4" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="212"/>
-      <c r="G4" s="212"/>
-      <c r="H4" s="212"/>
-      <c r="I4" s="198" t="s">
+      <c r="F4" s="182"/>
+      <c r="G4" s="182"/>
+      <c r="H4" s="182"/>
+      <c r="I4" s="183" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="198"/>
-      <c r="K4" s="198"/>
+      <c r="J4" s="183"/>
+      <c r="K4" s="183"/>
       <c r="L4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="4" t="str">
+      <c r="M4" s="4">
         <f>'Mileage Detail'!M4</f>
-        <v>DIESEL</v>
-      </c>
-      <c r="N4" s="212" t="s">
+        <v>0</v>
+      </c>
+      <c r="N4" s="182" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="203" t="s">
+      <c r="O4" s="184" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="202"/>
-      <c r="B5" s="202"/>
-      <c r="C5" s="211"/>
-      <c r="D5" s="211"/>
-      <c r="E5" s="212"/>
-      <c r="F5" s="212"/>
-      <c r="G5" s="212"/>
-      <c r="H5" s="212"/>
-      <c r="I5" s="198"/>
-      <c r="J5" s="198"/>
-      <c r="K5" s="198"/>
+      <c r="A5" s="180"/>
+      <c r="B5" s="180"/>
+      <c r="C5" s="181"/>
+      <c r="D5" s="181"/>
+      <c r="E5" s="182"/>
+      <c r="F5" s="182"/>
+      <c r="G5" s="182"/>
+      <c r="H5" s="182"/>
+      <c r="I5" s="183"/>
+      <c r="J5" s="183"/>
+      <c r="K5" s="183"/>
       <c r="L5" s="6" t="s">
         <v>7</v>
       </c>
       <c r="M5" s="7">
         <f>'Mileage Detail'!M5</f>
-        <v>1600</v>
-      </c>
-      <c r="N5" s="212"/>
-      <c r="O5" s="203"/>
+        <v>0</v>
+      </c>
+      <c r="N5" s="182"/>
+      <c r="O5" s="184"/>
     </row>
     <row r="6" spans="1:15" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="204" t="s">
+      <c r="A6" s="185" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="204"/>
-      <c r="C6" s="205"/>
-      <c r="D6" s="205"/>
-      <c r="E6" s="205" t="s">
-        <v>203</v>
-      </c>
-      <c r="F6" s="205"/>
-      <c r="G6" s="205"/>
-      <c r="H6" s="205"/>
-      <c r="I6" s="206"/>
-      <c r="J6" s="206"/>
-      <c r="K6" s="206"/>
-      <c r="L6" s="207" t="s">
+      <c r="B6" s="185"/>
+      <c r="C6" s="186"/>
+      <c r="D6" s="186"/>
+      <c r="E6" s="186"/>
+      <c r="F6" s="186"/>
+      <c r="G6" s="186"/>
+      <c r="H6" s="186"/>
+      <c r="I6" s="187"/>
+      <c r="J6" s="187"/>
+      <c r="K6" s="187"/>
+      <c r="L6" s="188" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="203" t="str">
+      <c r="M6" s="184">
         <f>'Mileage Detail'!M6</f>
-        <v>SB65 XCW</v>
-      </c>
-      <c r="N6" s="208">
+        <v>0</v>
+      </c>
+      <c r="N6" s="189">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
-      </c>
-      <c r="O6" s="203"/>
+        <v>46058</v>
+      </c>
+      <c r="O6" s="184"/>
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="204"/>
-      <c r="B7" s="204"/>
-      <c r="C7" s="205"/>
-      <c r="D7" s="205"/>
-      <c r="E7" s="205"/>
-      <c r="F7" s="205"/>
-      <c r="G7" s="205"/>
-      <c r="H7" s="205"/>
-      <c r="I7" s="206"/>
-      <c r="J7" s="206"/>
-      <c r="K7" s="206"/>
-      <c r="L7" s="207"/>
-      <c r="M7" s="207"/>
-      <c r="N7" s="208"/>
-      <c r="O7" s="203"/>
+      <c r="A7" s="185"/>
+      <c r="B7" s="185"/>
+      <c r="C7" s="186"/>
+      <c r="D7" s="186"/>
+      <c r="E7" s="186"/>
+      <c r="F7" s="186"/>
+      <c r="G7" s="186"/>
+      <c r="H7" s="186"/>
+      <c r="I7" s="187"/>
+      <c r="J7" s="187"/>
+      <c r="K7" s="187"/>
+      <c r="L7" s="188"/>
+      <c r="M7" s="188"/>
+      <c r="N7" s="189"/>
+      <c r="O7" s="184"/>
     </row>
     <row r="8" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="198" t="s">
+      <c r="A8" s="183" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="202" t="s">
+      <c r="B8" s="180" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="198" t="s">
+      <c r="C8" s="183" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="198"/>
-      <c r="E8" s="198" t="s">
+      <c r="D8" s="183"/>
+      <c r="E8" s="183" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="198" t="s">
+      <c r="F8" s="183" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="198" t="s">
+      <c r="G8" s="183" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="198" t="s">
+      <c r="H8" s="183" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="198" t="s">
+      <c r="I8" s="183" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="198" t="s">
+      <c r="J8" s="183" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="198" t="s">
+      <c r="K8" s="183" t="s">
         <v>19</v>
       </c>
-      <c r="L8" s="198" t="s">
+      <c r="L8" s="183" t="s">
         <v>20</v>
       </c>
-      <c r="M8" s="199" t="s">
+      <c r="M8" s="190" t="s">
         <v>21</v>
       </c>
-      <c r="N8" s="198" t="s">
+      <c r="N8" s="183" t="s">
         <v>22</v>
       </c>
-      <c r="O8" s="200" t="s">
+      <c r="O8" s="191" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="198"/>
-      <c r="B9" s="198"/>
-      <c r="C9" s="198"/>
-      <c r="D9" s="198"/>
-      <c r="E9" s="198"/>
-      <c r="F9" s="198"/>
-      <c r="G9" s="198"/>
-      <c r="H9" s="198"/>
-      <c r="I9" s="198"/>
-      <c r="J9" s="198"/>
-      <c r="K9" s="198"/>
-      <c r="L9" s="198"/>
-      <c r="M9" s="199"/>
-      <c r="N9" s="198"/>
-      <c r="O9" s="198"/>
+      <c r="A9" s="183"/>
+      <c r="B9" s="183"/>
+      <c r="C9" s="183"/>
+      <c r="D9" s="183"/>
+      <c r="E9" s="183"/>
+      <c r="F9" s="183"/>
+      <c r="G9" s="183"/>
+      <c r="H9" s="183"/>
+      <c r="I9" s="183"/>
+      <c r="J9" s="183"/>
+      <c r="K9" s="183"/>
+      <c r="L9" s="183"/>
+      <c r="M9" s="190"/>
+      <c r="N9" s="183"/>
+      <c r="O9" s="183"/>
     </row>
     <row r="10" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="198"/>
-      <c r="B10" s="198"/>
-      <c r="C10" s="198"/>
-      <c r="D10" s="198"/>
-      <c r="E10" s="198"/>
-      <c r="F10" s="198"/>
-      <c r="G10" s="198"/>
-      <c r="H10" s="198"/>
-      <c r="I10" s="198"/>
-      <c r="J10" s="198"/>
-      <c r="K10" s="198"/>
-      <c r="L10" s="198"/>
-      <c r="M10" s="199"/>
-      <c r="N10" s="198"/>
-      <c r="O10" s="198"/>
+      <c r="A10" s="183"/>
+      <c r="B10" s="183"/>
+      <c r="C10" s="183"/>
+      <c r="D10" s="183"/>
+      <c r="E10" s="183"/>
+      <c r="F10" s="183"/>
+      <c r="G10" s="183"/>
+      <c r="H10" s="183"/>
+      <c r="I10" s="183"/>
+      <c r="J10" s="183"/>
+      <c r="K10" s="183"/>
+      <c r="L10" s="183"/>
+      <c r="M10" s="190"/>
+      <c r="N10" s="183"/>
+      <c r="O10" s="183"/>
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="8"/>
@@ -3990,10 +3971,10 @@
       <c r="B43" s="42"/>
       <c r="E43" s="42"/>
       <c r="F43" s="42"/>
-      <c r="G43" s="201" t="s">
+      <c r="G43" s="192" t="s">
         <v>34</v>
       </c>
-      <c r="H43" s="201"/>
+      <c r="H43" s="192"/>
       <c r="I43" s="43"/>
       <c r="J43" s="43"/>
       <c r="K43" s="43"/>
@@ -4005,13 +3986,13 @@
       <c r="O43" s="44"/>
     </row>
     <row r="44" spans="1:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B44" s="192">
+      <c r="B44" s="193">
         <f>IF(OR(B49="no",AND(B49="yes",B54=0.25)),0,"WARNING - NON COMPANY CAR USERS WHO HAVE CLAIMED OVER 10,000 BUSINESS MILES IN A TAX YEAR MUST USE A CLAIM PER MILE RATE OF 25p")</f>
         <v>0</v>
       </c>
-      <c r="C44" s="192"/>
-      <c r="D44" s="192"/>
-      <c r="E44" s="192"/>
+      <c r="C44" s="193"/>
+      <c r="D44" s="193"/>
+      <c r="E44" s="193"/>
       <c r="F44" s="42"/>
       <c r="G44" s="45" t="s">
         <v>36</v>
@@ -4037,18 +4018,18 @@
       <c r="N44" s="47">
         <v>95195</v>
       </c>
-      <c r="O44" s="193" t="s">
+      <c r="O44" s="194" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="41"/>
-      <c r="B45" s="192"/>
-      <c r="C45" s="192"/>
-      <c r="D45" s="192"/>
-      <c r="E45" s="192"/>
+      <c r="B45" s="193"/>
+      <c r="C45" s="193"/>
+      <c r="D45" s="193"/>
+      <c r="E45" s="193"/>
       <c r="F45" s="42"/>
-      <c r="G45" s="194">
+      <c r="G45" s="195">
         <f>+G42-H42-SUM(I56,J56,K58,L56,M56,N56)</f>
         <v>0</v>
       </c>
@@ -4067,7 +4048,7 @@
       <c r="N45" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="O45" s="193"/>
+      <c r="O45" s="194"/>
     </row>
     <row r="46" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="41"/>
@@ -4076,7 +4057,7 @@
       <c r="D46" s="50"/>
       <c r="E46" s="50"/>
       <c r="F46" s="42"/>
-      <c r="G46" s="194"/>
+      <c r="G46" s="195"/>
       <c r="H46" s="46"/>
       <c r="I46" s="47"/>
       <c r="J46" s="47"/>
@@ -4092,7 +4073,7 @@
       </c>
       <c r="E47" s="51"/>
       <c r="F47" s="42"/>
-      <c r="G47" s="194"/>
+      <c r="G47" s="195"/>
       <c r="H47" s="46" t="s">
         <v>42</v>
       </c>
@@ -4131,19 +4112,19 @@
       <c r="O48" s="56"/>
     </row>
     <row r="49" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A49" s="184" t="s">
+      <c r="A49" s="196" t="s">
         <v>43</v>
       </c>
-      <c r="B49" s="195" t="s">
+      <c r="B49" s="197" t="s">
         <v>77</v>
       </c>
-      <c r="C49" s="196" t="s">
+      <c r="C49" s="198" t="s">
         <v>45</v>
       </c>
-      <c r="D49" s="196"/>
-      <c r="E49" s="196"/>
-      <c r="F49" s="196"/>
-      <c r="G49" s="197" t="s">
+      <c r="D49" s="198"/>
+      <c r="E49" s="198"/>
+      <c r="F49" s="198"/>
+      <c r="G49" s="199" t="s">
         <v>46</v>
       </c>
       <c r="H49" s="43" t="s">
@@ -4178,13 +4159,13 @@
       </c>
     </row>
     <row r="50" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A50" s="184"/>
-      <c r="B50" s="195"/>
-      <c r="C50" s="196"/>
-      <c r="D50" s="196"/>
-      <c r="E50" s="196"/>
-      <c r="F50" s="196"/>
-      <c r="G50" s="197"/>
+      <c r="A50" s="196"/>
+      <c r="B50" s="197"/>
+      <c r="C50" s="198"/>
+      <c r="D50" s="198"/>
+      <c r="E50" s="198"/>
+      <c r="F50" s="198"/>
+      <c r="G50" s="199"/>
       <c r="H50" s="23"/>
       <c r="I50" s="61"/>
       <c r="J50" s="61"/>
@@ -4195,20 +4176,20 @@
       <c r="O50" s="52"/>
     </row>
     <row r="51" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A51" s="184" t="s">
+      <c r="A51" s="196" t="s">
         <v>48</v>
       </c>
-      <c r="B51" s="185">
+      <c r="B51" s="204">
         <f>'Mileage Detail'!E37</f>
         <v>0</v>
       </c>
-      <c r="C51" s="186" t="s">
+      <c r="C51" s="205" t="s">
         <v>49</v>
       </c>
-      <c r="D51" s="186"/>
-      <c r="E51" s="186"/>
-      <c r="F51" s="186"/>
-      <c r="G51" s="187" t="s">
+      <c r="D51" s="205"/>
+      <c r="E51" s="205"/>
+      <c r="F51" s="205"/>
+      <c r="G51" s="206" t="s">
         <v>50</v>
       </c>
       <c r="H51" s="23" t="s">
@@ -4229,13 +4210,13 @@
       </c>
     </row>
     <row r="52" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A52" s="184"/>
-      <c r="B52" s="184"/>
-      <c r="C52" s="186"/>
-      <c r="D52" s="186"/>
-      <c r="E52" s="186"/>
-      <c r="F52" s="186"/>
-      <c r="G52" s="187"/>
+      <c r="A52" s="196"/>
+      <c r="B52" s="196"/>
+      <c r="C52" s="205"/>
+      <c r="D52" s="205"/>
+      <c r="E52" s="205"/>
+      <c r="F52" s="205"/>
+      <c r="G52" s="206"/>
       <c r="H52" s="23" t="s">
         <v>52</v>
       </c>
@@ -4260,11 +4241,11 @@
       <c r="B53" s="64">
         <v>0.45</v>
       </c>
-      <c r="C53" s="186"/>
-      <c r="D53" s="186"/>
-      <c r="E53" s="186"/>
-      <c r="F53" s="186"/>
-      <c r="G53" s="187"/>
+      <c r="C53" s="205"/>
+      <c r="D53" s="205"/>
+      <c r="E53" s="205"/>
+      <c r="F53" s="205"/>
+      <c r="G53" s="206"/>
       <c r="H53" s="23" t="s">
         <v>54</v>
       </c>
@@ -4295,20 +4276,20 @@
       </c>
     </row>
     <row r="54" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A54" s="188" t="s">
+      <c r="A54" s="207" t="s">
         <v>55</v>
       </c>
-      <c r="B54" s="189">
+      <c r="B54" s="208">
         <f>B51*B53</f>
         <v>0</v>
       </c>
-      <c r="C54" s="190" t="s">
+      <c r="C54" s="209" t="s">
         <v>56</v>
       </c>
-      <c r="D54" s="190"/>
-      <c r="E54" s="190"/>
-      <c r="F54" s="190"/>
-      <c r="G54" s="187"/>
+      <c r="D54" s="209"/>
+      <c r="E54" s="209"/>
+      <c r="F54" s="209"/>
+      <c r="G54" s="206"/>
       <c r="H54" s="23" t="s">
         <v>57</v>
       </c>
@@ -4339,13 +4320,13 @@
       </c>
     </row>
     <row r="55" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A55" s="188"/>
-      <c r="B55" s="188"/>
-      <c r="C55" s="190"/>
-      <c r="D55" s="190"/>
-      <c r="E55" s="190"/>
-      <c r="F55" s="190"/>
-      <c r="G55" s="187"/>
+      <c r="A55" s="207"/>
+      <c r="B55" s="207"/>
+      <c r="C55" s="209"/>
+      <c r="D55" s="209"/>
+      <c r="E55" s="209"/>
+      <c r="F55" s="209"/>
+      <c r="G55" s="206"/>
       <c r="H55" s="23" t="s">
         <v>58</v>
       </c>
@@ -4379,7 +4360,7 @@
       <c r="A56" s="42"/>
       <c r="B56" s="66"/>
       <c r="E56" s="51"/>
-      <c r="G56" s="187"/>
+      <c r="G56" s="206"/>
       <c r="H56" s="23" t="s">
         <v>47</v>
       </c>
@@ -4415,10 +4396,10 @@
     <row r="57" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="68"/>
       <c r="B57" s="69"/>
-      <c r="C57" s="191"/>
-      <c r="D57" s="191"/>
+      <c r="C57" s="210"/>
+      <c r="D57" s="210"/>
       <c r="E57" s="70"/>
-      <c r="G57" s="187"/>
+      <c r="G57" s="206"/>
       <c r="H57" s="71" t="s">
         <v>59</v>
       </c>
@@ -4470,13 +4451,13 @@
       <c r="D59" s="42"/>
     </row>
     <row r="60" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B60" s="180" t="s">
+      <c r="B60" s="212" t="s">
         <v>60</v>
       </c>
-      <c r="C60" s="180"/>
-      <c r="D60" s="180"/>
-      <c r="E60" s="180"/>
-      <c r="F60" s="180"/>
+      <c r="C60" s="212"/>
+      <c r="D60" s="212"/>
+      <c r="E60" s="212"/>
+      <c r="F60" s="212"/>
       <c r="G60" s="80"/>
       <c r="H60" s="81"/>
       <c r="I60" s="81"/>
@@ -4502,10 +4483,10 @@
       <c r="K61" s="88"/>
       <c r="L61" s="88"/>
       <c r="M61" s="88"/>
-      <c r="N61" s="181" t="s">
+      <c r="N61" s="200" t="s">
         <v>62</v>
       </c>
-      <c r="O61" s="181"/>
+      <c r="O61" s="200"/>
     </row>
     <row r="62" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62" s="89"/>
@@ -4520,8 +4501,8 @@
       <c r="K62" s="88"/>
       <c r="L62" s="88"/>
       <c r="M62" s="92"/>
-      <c r="N62" s="181"/>
-      <c r="O62" s="181"/>
+      <c r="N62" s="200"/>
+      <c r="O62" s="200"/>
     </row>
     <row r="63" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B63" s="89"/>
@@ -4529,21 +4510,21 @@
         <v>63</v>
       </c>
       <c r="D63" s="93"/>
-      <c r="E63" s="182"/>
-      <c r="F63" s="182"/>
+      <c r="E63" s="201"/>
+      <c r="F63" s="201"/>
       <c r="G63" s="91"/>
       <c r="H63" s="94" t="s">
         <v>64</v>
       </c>
-      <c r="I63" s="183"/>
-      <c r="J63" s="183"/>
-      <c r="K63" s="183"/>
+      <c r="I63" s="202"/>
+      <c r="J63" s="202"/>
+      <c r="K63" s="202"/>
       <c r="L63" s="96" t="s">
         <v>11</v>
       </c>
       <c r="M63" s="95"/>
-      <c r="N63" s="181"/>
-      <c r="O63" s="181"/>
+      <c r="N63" s="200"/>
+      <c r="O63" s="200"/>
     </row>
     <row r="64" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B64" s="89"/>
@@ -4733,10 +4714,10 @@
       <c r="E74" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F74" s="178" t="s">
+      <c r="F74" s="203" t="s">
         <v>76</v>
       </c>
-      <c r="G74" s="178"/>
+      <c r="G74" s="203"/>
       <c r="H74" s="116"/>
       <c r="I74" s="114"/>
       <c r="J74" s="70"/>
@@ -4759,10 +4740,10 @@
       <c r="E75" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F75" s="178" t="s">
+      <c r="F75" s="203" t="s">
         <v>80</v>
       </c>
-      <c r="G75" s="178"/>
+      <c r="G75" s="203"/>
       <c r="H75" s="5"/>
       <c r="I75" s="114"/>
       <c r="J75" s="70"/>
@@ -4783,10 +4764,10 @@
       <c r="E76" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F76" s="178" t="s">
+      <c r="F76" s="203" t="s">
         <v>83</v>
       </c>
-      <c r="G76" s="178"/>
+      <c r="G76" s="203"/>
       <c r="H76" s="5"/>
       <c r="I76" s="114"/>
       <c r="J76" s="70"/>
@@ -4807,10 +4788,10 @@
       <c r="E77" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F77" s="179" t="s">
+      <c r="F77" s="211" t="s">
         <v>86</v>
       </c>
-      <c r="G77" s="179"/>
+      <c r="G77" s="211"/>
       <c r="H77" s="114"/>
       <c r="I77" s="114"/>
       <c r="J77" s="70"/>
@@ -4834,10 +4815,10 @@
       <c r="E78" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F78" s="178" t="s">
+      <c r="F78" s="203" t="s">
         <v>89</v>
       </c>
-      <c r="G78" s="178"/>
+      <c r="G78" s="203"/>
       <c r="H78" s="114"/>
       <c r="I78" s="114"/>
       <c r="J78" s="70"/>
@@ -4932,43 +4913,11 @@
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="A1:G3"/>
-    <mergeCell ref="H1:N3"/>
-    <mergeCell ref="A4:B5"/>
-    <mergeCell ref="C4:D5"/>
-    <mergeCell ref="E4:H5"/>
-    <mergeCell ref="I4:K5"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="O4:O7"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="C6:D7"/>
-    <mergeCell ref="E6:H7"/>
-    <mergeCell ref="I6:K7"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="N8:N10"/>
-    <mergeCell ref="O8:O10"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G8:G10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="B44:E45"/>
-    <mergeCell ref="O44:O45"/>
-    <mergeCell ref="G45:G47"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:F50"/>
-    <mergeCell ref="G49:G50"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="B60:F60"/>
     <mergeCell ref="N61:O63"/>
     <mergeCell ref="E63:F63"/>
     <mergeCell ref="I63:K63"/>
@@ -4981,11 +4930,43 @@
     <mergeCell ref="B54:B55"/>
     <mergeCell ref="C54:F55"/>
     <mergeCell ref="C57:D57"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="F77:G77"/>
-    <mergeCell ref="F78:G78"/>
-    <mergeCell ref="B60:F60"/>
+    <mergeCell ref="B44:E45"/>
+    <mergeCell ref="O44:O45"/>
+    <mergeCell ref="G45:G47"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:F50"/>
+    <mergeCell ref="G49:G50"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="N8:N10"/>
+    <mergeCell ref="O8:O10"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="O4:O7"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="C6:D7"/>
+    <mergeCell ref="E6:H7"/>
+    <mergeCell ref="I6:K7"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="H1:N3"/>
+    <mergeCell ref="A4:B5"/>
+    <mergeCell ref="C4:D5"/>
+    <mergeCell ref="E4:H5"/>
+    <mergeCell ref="I4:K5"/>
+    <mergeCell ref="N4:N5"/>
   </mergeCells>
   <conditionalFormatting sqref="B44">
     <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Warning">
@@ -5048,246 +5029,246 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="209" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="209"/>
-      <c r="C1" s="209"/>
-      <c r="D1" s="209"/>
-      <c r="E1" s="209"/>
-      <c r="F1" s="209"/>
-      <c r="G1" s="209"/>
-      <c r="H1" s="210"/>
-      <c r="I1" s="210"/>
-      <c r="J1" s="210"/>
-      <c r="K1" s="210"/>
-      <c r="L1" s="210"/>
-      <c r="M1" s="210"/>
-      <c r="N1" s="210"/>
+      <c r="A1" s="178" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="178"/>
+      <c r="C1" s="178"/>
+      <c r="D1" s="178"/>
+      <c r="E1" s="178"/>
+      <c r="F1" s="178"/>
+      <c r="G1" s="178"/>
+      <c r="H1" s="179"/>
+      <c r="I1" s="179"/>
+      <c r="J1" s="179"/>
+      <c r="K1" s="179"/>
+      <c r="L1" s="179"/>
+      <c r="M1" s="179"/>
+      <c r="N1" s="179"/>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="209"/>
-      <c r="B2" s="209"/>
-      <c r="C2" s="209"/>
-      <c r="D2" s="209"/>
-      <c r="E2" s="209"/>
-      <c r="F2" s="209"/>
-      <c r="G2" s="209"/>
-      <c r="H2" s="210"/>
-      <c r="I2" s="210"/>
-      <c r="J2" s="210"/>
-      <c r="K2" s="210"/>
-      <c r="L2" s="210"/>
-      <c r="M2" s="210"/>
-      <c r="N2" s="210"/>
+      <c r="A2" s="178"/>
+      <c r="B2" s="178"/>
+      <c r="C2" s="178"/>
+      <c r="D2" s="178"/>
+      <c r="E2" s="178"/>
+      <c r="F2" s="178"/>
+      <c r="G2" s="178"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
+      <c r="L2" s="179"/>
+      <c r="M2" s="179"/>
+      <c r="N2" s="179"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="209"/>
-      <c r="B3" s="209"/>
-      <c r="C3" s="209"/>
-      <c r="D3" s="209"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="209"/>
-      <c r="G3" s="209"/>
-      <c r="H3" s="210"/>
-      <c r="I3" s="210"/>
-      <c r="J3" s="210"/>
-      <c r="K3" s="210"/>
-      <c r="L3" s="210"/>
-      <c r="M3" s="210"/>
-      <c r="N3" s="210"/>
+      <c r="A3" s="178"/>
+      <c r="B3" s="178"/>
+      <c r="C3" s="178"/>
+      <c r="D3" s="178"/>
+      <c r="E3" s="178"/>
+      <c r="F3" s="178"/>
+      <c r="G3" s="178"/>
+      <c r="H3" s="179"/>
+      <c r="I3" s="179"/>
+      <c r="J3" s="179"/>
+      <c r="K3" s="179"/>
+      <c r="L3" s="179"/>
+      <c r="M3" s="179"/>
+      <c r="N3" s="179"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="202" t="s">
+      <c r="A4" s="180" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="202"/>
-      <c r="C4" s="216" t="str">
+      <c r="B4" s="180"/>
+      <c r="C4" s="213">
         <f>'Expense Claim Form '!C4:D5</f>
-        <v>Brian Fleming</v>
-      </c>
-      <c r="D4" s="216"/>
-      <c r="E4" s="212" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="213"/>
+      <c r="E4" s="182" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="212"/>
-      <c r="G4" s="212"/>
-      <c r="H4" s="212"/>
-      <c r="I4" s="198" t="s">
+      <c r="F4" s="182"/>
+      <c r="G4" s="182"/>
+      <c r="H4" s="182"/>
+      <c r="I4" s="183" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="198"/>
-      <c r="K4" s="198"/>
+      <c r="J4" s="183"/>
+      <c r="K4" s="183"/>
       <c r="L4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="4" t="str">
+      <c r="M4" s="4">
         <f>'Mileage Detail'!M4</f>
-        <v>DIESEL</v>
-      </c>
-      <c r="N4" s="212" t="s">
+        <v>0</v>
+      </c>
+      <c r="N4" s="182" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="203" t="s">
+      <c r="O4" s="184" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="202"/>
-      <c r="B5" s="202"/>
-      <c r="C5" s="216"/>
-      <c r="D5" s="216"/>
-      <c r="E5" s="212"/>
-      <c r="F5" s="212"/>
-      <c r="G5" s="212"/>
-      <c r="H5" s="212"/>
-      <c r="I5" s="198"/>
-      <c r="J5" s="198"/>
-      <c r="K5" s="198"/>
+      <c r="A5" s="180"/>
+      <c r="B5" s="180"/>
+      <c r="C5" s="213"/>
+      <c r="D5" s="213"/>
+      <c r="E5" s="182"/>
+      <c r="F5" s="182"/>
+      <c r="G5" s="182"/>
+      <c r="H5" s="182"/>
+      <c r="I5" s="183"/>
+      <c r="J5" s="183"/>
+      <c r="K5" s="183"/>
       <c r="L5" s="6" t="s">
         <v>7</v>
       </c>
       <c r="M5" s="7">
         <f>'Mileage Detail'!M5</f>
-        <v>1600</v>
-      </c>
-      <c r="N5" s="212"/>
-      <c r="O5" s="203"/>
+        <v>0</v>
+      </c>
+      <c r="N5" s="182"/>
+      <c r="O5" s="184"/>
     </row>
     <row r="6" spans="1:15" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="204" t="s">
+      <c r="A6" s="185" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="204"/>
-      <c r="C6" s="216">
+      <c r="B6" s="185"/>
+      <c r="C6" s="213">
         <f>'Expense Claim Form '!C6:D7</f>
         <v>0</v>
       </c>
-      <c r="D6" s="216"/>
-      <c r="E6" s="216" t="str">
+      <c r="D6" s="213"/>
+      <c r="E6" s="213">
         <f>'Expense Claim Form '!E6:H7</f>
-        <v>Taylor Wimpey West of Scotland</v>
-      </c>
-      <c r="F6" s="216"/>
-      <c r="G6" s="216"/>
-      <c r="H6" s="216"/>
-      <c r="I6" s="203">
+        <v>0</v>
+      </c>
+      <c r="F6" s="213"/>
+      <c r="G6" s="213"/>
+      <c r="H6" s="213"/>
+      <c r="I6" s="184">
         <f>'Expense Claim Form '!I6:K7</f>
         <v>0</v>
       </c>
-      <c r="J6" s="203"/>
-      <c r="K6" s="203"/>
-      <c r="L6" s="207" t="s">
+      <c r="J6" s="184"/>
+      <c r="K6" s="184"/>
+      <c r="L6" s="188" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="203" t="str">
+      <c r="M6" s="184">
         <f>'Mileage Detail'!M6</f>
-        <v>SB65 XCW</v>
-      </c>
-      <c r="N6" s="208">
+        <v>0</v>
+      </c>
+      <c r="N6" s="189">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
-      </c>
-      <c r="O6" s="203"/>
+        <v>46058</v>
+      </c>
+      <c r="O6" s="184"/>
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="204"/>
-      <c r="B7" s="204"/>
-      <c r="C7" s="216"/>
-      <c r="D7" s="216"/>
-      <c r="E7" s="216"/>
-      <c r="F7" s="216"/>
-      <c r="G7" s="216"/>
-      <c r="H7" s="216"/>
-      <c r="I7" s="203"/>
-      <c r="J7" s="203"/>
-      <c r="K7" s="203"/>
-      <c r="L7" s="207"/>
-      <c r="M7" s="207"/>
-      <c r="N7" s="208"/>
-      <c r="O7" s="203"/>
+      <c r="A7" s="185"/>
+      <c r="B7" s="185"/>
+      <c r="C7" s="213"/>
+      <c r="D7" s="213"/>
+      <c r="E7" s="213"/>
+      <c r="F7" s="213"/>
+      <c r="G7" s="213"/>
+      <c r="H7" s="213"/>
+      <c r="I7" s="184"/>
+      <c r="J7" s="184"/>
+      <c r="K7" s="184"/>
+      <c r="L7" s="188"/>
+      <c r="M7" s="188"/>
+      <c r="N7" s="189"/>
+      <c r="O7" s="184"/>
     </row>
     <row r="8" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="198" t="s">
+      <c r="A8" s="183" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="202" t="s">
+      <c r="B8" s="180" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="198" t="s">
+      <c r="C8" s="183" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="198"/>
-      <c r="E8" s="198" t="s">
+      <c r="D8" s="183"/>
+      <c r="E8" s="183" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="198" t="s">
+      <c r="F8" s="183" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="198" t="s">
+      <c r="G8" s="183" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="198" t="s">
+      <c r="H8" s="183" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="198" t="s">
+      <c r="I8" s="183" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="198" t="s">
+      <c r="J8" s="183" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="198" t="s">
+      <c r="K8" s="183" t="s">
         <v>19</v>
       </c>
-      <c r="L8" s="198" t="s">
+      <c r="L8" s="183" t="s">
         <v>20</v>
       </c>
-      <c r="M8" s="199" t="s">
+      <c r="M8" s="190" t="s">
         <v>21</v>
       </c>
-      <c r="N8" s="198" t="s">
+      <c r="N8" s="183" t="s">
         <v>22</v>
       </c>
-      <c r="O8" s="200" t="s">
+      <c r="O8" s="191" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="198"/>
-      <c r="B9" s="198"/>
-      <c r="C9" s="198"/>
-      <c r="D9" s="198"/>
-      <c r="E9" s="198"/>
-      <c r="F9" s="198"/>
-      <c r="G9" s="198"/>
-      <c r="H9" s="198"/>
-      <c r="I9" s="198"/>
-      <c r="J9" s="198"/>
-      <c r="K9" s="198"/>
-      <c r="L9" s="198"/>
-      <c r="M9" s="199"/>
-      <c r="N9" s="198"/>
-      <c r="O9" s="198"/>
+      <c r="A9" s="183"/>
+      <c r="B9" s="183"/>
+      <c r="C9" s="183"/>
+      <c r="D9" s="183"/>
+      <c r="E9" s="183"/>
+      <c r="F9" s="183"/>
+      <c r="G9" s="183"/>
+      <c r="H9" s="183"/>
+      <c r="I9" s="183"/>
+      <c r="J9" s="183"/>
+      <c r="K9" s="183"/>
+      <c r="L9" s="183"/>
+      <c r="M9" s="190"/>
+      <c r="N9" s="183"/>
+      <c r="O9" s="183"/>
     </row>
     <row r="10" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="198"/>
-      <c r="B10" s="198"/>
-      <c r="C10" s="198"/>
-      <c r="D10" s="198"/>
-      <c r="E10" s="198"/>
-      <c r="F10" s="198"/>
-      <c r="G10" s="198"/>
-      <c r="H10" s="198"/>
-      <c r="I10" s="198"/>
-      <c r="J10" s="198"/>
-      <c r="K10" s="198"/>
-      <c r="L10" s="198"/>
-      <c r="M10" s="199"/>
-      <c r="N10" s="198"/>
-      <c r="O10" s="198"/>
+      <c r="A10" s="183"/>
+      <c r="B10" s="183"/>
+      <c r="C10" s="183"/>
+      <c r="D10" s="183"/>
+      <c r="E10" s="183"/>
+      <c r="F10" s="183"/>
+      <c r="G10" s="183"/>
+      <c r="H10" s="183"/>
+      <c r="I10" s="183"/>
+      <c r="J10" s="183"/>
+      <c r="K10" s="183"/>
+      <c r="L10" s="183"/>
+      <c r="M10" s="190"/>
+      <c r="N10" s="183"/>
+      <c r="O10" s="183"/>
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="8"/>
@@ -6918,10 +6899,10 @@
       <c r="B53" s="42"/>
       <c r="E53" s="42"/>
       <c r="F53" s="42"/>
-      <c r="G53" s="201" t="s">
+      <c r="G53" s="192" t="s">
         <v>34</v>
       </c>
-      <c r="H53" s="201"/>
+      <c r="H53" s="192"/>
       <c r="I53" s="43"/>
       <c r="J53" s="43"/>
       <c r="K53" s="43"/>
@@ -6933,10 +6914,10 @@
       <c r="O53" s="44"/>
     </row>
     <row r="54" spans="1:15" ht="34.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B54" s="213"/>
-      <c r="C54" s="213"/>
-      <c r="D54" s="213"/>
-      <c r="E54" s="213"/>
+      <c r="B54" s="214"/>
+      <c r="C54" s="214"/>
+      <c r="D54" s="214"/>
+      <c r="E54" s="214"/>
       <c r="G54" s="45" t="s">
         <v>36</v>
       </c>
@@ -6961,16 +6942,16 @@
       <c r="N54" s="47">
         <v>95195</v>
       </c>
-      <c r="O54" s="193" t="s">
+      <c r="O54" s="194" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="55" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B55" s="213"/>
-      <c r="C55" s="213"/>
-      <c r="D55" s="213"/>
-      <c r="E55" s="213"/>
-      <c r="G55" s="194">
+      <c r="B55" s="214"/>
+      <c r="C55" s="214"/>
+      <c r="D55" s="214"/>
+      <c r="E55" s="214"/>
+      <c r="G55" s="195">
         <f>+G52-H52-SUM(I66:N66)</f>
         <v>0</v>
       </c>
@@ -6989,7 +6970,7 @@
       <c r="N55" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="O55" s="193"/>
+      <c r="O55" s="194"/>
     </row>
     <row r="56" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="41"/>
@@ -6998,7 +6979,7 @@
       <c r="D56" s="50"/>
       <c r="E56" s="50"/>
       <c r="F56" s="42"/>
-      <c r="G56" s="194"/>
+      <c r="G56" s="195"/>
       <c r="H56" s="46"/>
       <c r="I56" s="47"/>
       <c r="J56" s="47"/>
@@ -7009,7 +6990,7 @@
       <c r="O56" s="48"/>
     </row>
     <row r="57" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G57" s="194"/>
+      <c r="G57" s="195"/>
       <c r="H57" s="46" t="s">
         <v>42</v>
       </c>
@@ -7045,13 +7026,13 @@
       <c r="O58" s="56"/>
     </row>
     <row r="59" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A59" s="213"/>
-      <c r="B59" s="213"/>
-      <c r="C59" s="213"/>
-      <c r="D59" s="213"/>
-      <c r="E59" s="213"/>
-      <c r="F59" s="213"/>
-      <c r="G59" s="197" t="s">
+      <c r="A59" s="214"/>
+      <c r="B59" s="214"/>
+      <c r="C59" s="214"/>
+      <c r="D59" s="214"/>
+      <c r="E59" s="214"/>
+      <c r="F59" s="214"/>
+      <c r="G59" s="199" t="s">
         <v>46</v>
       </c>
       <c r="H59" s="43" t="s">
@@ -7086,13 +7067,13 @@
       </c>
     </row>
     <row r="60" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A60" s="213"/>
-      <c r="B60" s="213"/>
-      <c r="C60" s="213"/>
-      <c r="D60" s="213"/>
-      <c r="E60" s="213"/>
-      <c r="F60" s="213"/>
-      <c r="G60" s="197"/>
+      <c r="A60" s="214"/>
+      <c r="B60" s="214"/>
+      <c r="C60" s="214"/>
+      <c r="D60" s="214"/>
+      <c r="E60" s="214"/>
+      <c r="F60" s="214"/>
+      <c r="G60" s="199"/>
       <c r="H60" s="23"/>
       <c r="I60" s="21"/>
       <c r="J60" s="21"/>
@@ -7103,13 +7084,13 @@
       <c r="O60" s="52"/>
     </row>
     <row r="61" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A61" s="213"/>
-      <c r="B61" s="214"/>
-      <c r="C61" s="213"/>
-      <c r="D61" s="213"/>
-      <c r="E61" s="213"/>
-      <c r="F61" s="213"/>
-      <c r="G61" s="215" t="s">
+      <c r="A61" s="214"/>
+      <c r="B61" s="215"/>
+      <c r="C61" s="214"/>
+      <c r="D61" s="214"/>
+      <c r="E61" s="214"/>
+      <c r="F61" s="214"/>
+      <c r="G61" s="216" t="s">
         <v>50</v>
       </c>
       <c r="H61" s="23" t="s">
@@ -7130,13 +7111,13 @@
       </c>
     </row>
     <row r="62" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A62" s="213"/>
-      <c r="B62" s="213"/>
-      <c r="C62" s="213"/>
-      <c r="D62" s="213"/>
-      <c r="E62" s="213"/>
-      <c r="F62" s="213"/>
-      <c r="G62" s="215"/>
+      <c r="A62" s="214"/>
+      <c r="B62" s="214"/>
+      <c r="C62" s="214"/>
+      <c r="D62" s="214"/>
+      <c r="E62" s="214"/>
+      <c r="F62" s="214"/>
+      <c r="G62" s="216"/>
       <c r="H62" s="23" t="s">
         <v>52</v>
       </c>
@@ -7156,11 +7137,11 @@
     </row>
     <row r="63" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B63"/>
-      <c r="C63" s="213"/>
-      <c r="D63" s="213"/>
-      <c r="E63" s="213"/>
-      <c r="F63" s="213"/>
-      <c r="G63" s="215"/>
+      <c r="C63" s="214"/>
+      <c r="D63" s="214"/>
+      <c r="E63" s="214"/>
+      <c r="F63" s="214"/>
+      <c r="G63" s="216"/>
       <c r="H63" s="23" t="s">
         <v>54</v>
       </c>
@@ -7191,13 +7172,13 @@
       </c>
     </row>
     <row r="64" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A64" s="213"/>
-      <c r="B64" s="214"/>
-      <c r="C64" s="213"/>
-      <c r="D64" s="213"/>
-      <c r="E64" s="213"/>
-      <c r="F64" s="213"/>
-      <c r="G64" s="215"/>
+      <c r="A64" s="214"/>
+      <c r="B64" s="215"/>
+      <c r="C64" s="214"/>
+      <c r="D64" s="214"/>
+      <c r="E64" s="214"/>
+      <c r="F64" s="214"/>
+      <c r="G64" s="216"/>
       <c r="H64" s="23" t="s">
         <v>57</v>
       </c>
@@ -7228,13 +7209,13 @@
       </c>
     </row>
     <row r="65" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A65" s="213"/>
-      <c r="B65" s="213"/>
-      <c r="C65" s="213"/>
-      <c r="D65" s="213"/>
-      <c r="E65" s="213"/>
-      <c r="F65" s="213"/>
-      <c r="G65" s="215"/>
+      <c r="A65" s="214"/>
+      <c r="B65" s="214"/>
+      <c r="C65" s="214"/>
+      <c r="D65" s="214"/>
+      <c r="E65" s="214"/>
+      <c r="F65" s="214"/>
+      <c r="G65" s="216"/>
       <c r="H65" s="23" t="s">
         <v>58</v>
       </c>
@@ -7265,7 +7246,7 @@
       </c>
     </row>
     <row r="66" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G66" s="215"/>
+      <c r="G66" s="216"/>
       <c r="H66" s="23" t="s">
         <v>47</v>
       </c>
@@ -7300,9 +7281,9 @@
     </row>
     <row r="67" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B67"/>
-      <c r="C67" s="213"/>
-      <c r="D67" s="213"/>
-      <c r="G67" s="215"/>
+      <c r="C67" s="214"/>
+      <c r="D67" s="214"/>
+      <c r="G67" s="216"/>
       <c r="H67" s="54" t="s">
         <v>59</v>
       </c>
@@ -7403,10 +7384,10 @@
       <c r="E72" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F72" s="178" t="s">
+      <c r="F72" s="203" t="s">
         <v>76</v>
       </c>
-      <c r="G72" s="178"/>
+      <c r="G72" s="203"/>
       <c r="H72" s="116"/>
       <c r="I72" s="114"/>
       <c r="J72" s="70"/>
@@ -7429,10 +7410,10 @@
       <c r="E73" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F73" s="178" t="s">
+      <c r="F73" s="203" t="s">
         <v>80</v>
       </c>
-      <c r="G73" s="178"/>
+      <c r="G73" s="203"/>
       <c r="H73" s="5"/>
       <c r="I73" s="114"/>
       <c r="J73" s="70"/>
@@ -7453,10 +7434,10 @@
       <c r="E74" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="F74" s="178" t="s">
+      <c r="F74" s="203" t="s">
         <v>83</v>
       </c>
-      <c r="G74" s="178"/>
+      <c r="G74" s="203"/>
       <c r="H74" s="5"/>
       <c r="I74" s="114"/>
       <c r="J74" s="70"/>
@@ -7477,10 +7458,10 @@
       <c r="E75" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F75" s="179" t="s">
+      <c r="F75" s="211" t="s">
         <v>86</v>
       </c>
-      <c r="G75" s="179"/>
+      <c r="G75" s="211"/>
       <c r="H75" s="114"/>
       <c r="I75" s="114"/>
       <c r="J75" s="70"/>
@@ -7504,10 +7485,10 @@
       <c r="E76" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F76" s="178" t="s">
+      <c r="F76" s="203" t="s">
         <v>89</v>
       </c>
-      <c r="G76" s="178"/>
+      <c r="G76" s="203"/>
       <c r="H76" s="114"/>
       <c r="I76" s="114"/>
       <c r="J76" s="70"/>
@@ -7565,26 +7546,26 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="A1:G3"/>
-    <mergeCell ref="H1:N3"/>
-    <mergeCell ref="A4:B5"/>
-    <mergeCell ref="C4:D5"/>
-    <mergeCell ref="E4:H5"/>
-    <mergeCell ref="I4:K5"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="O4:O7"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="C6:D7"/>
-    <mergeCell ref="E6:H7"/>
-    <mergeCell ref="I6:K7"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="C61:F63"/>
+    <mergeCell ref="G61:G67"/>
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:F65"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="B54:E55"/>
+    <mergeCell ref="O54:O55"/>
+    <mergeCell ref="G55:G57"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:F60"/>
+    <mergeCell ref="G59:G60"/>
     <mergeCell ref="L8:L10"/>
     <mergeCell ref="M8:M10"/>
     <mergeCell ref="N8:N10"/>
@@ -7595,26 +7576,26 @@
     <mergeCell ref="I8:I10"/>
     <mergeCell ref="J8:J10"/>
     <mergeCell ref="K8:K10"/>
-    <mergeCell ref="B54:E55"/>
-    <mergeCell ref="O54:O55"/>
-    <mergeCell ref="G55:G57"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:F60"/>
-    <mergeCell ref="G59:G60"/>
-    <mergeCell ref="A61:A62"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="C61:F63"/>
-    <mergeCell ref="G61:G67"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:F65"/>
-    <mergeCell ref="C67:D67"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="F73:G73"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="O4:O7"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="C6:D7"/>
+    <mergeCell ref="E6:H7"/>
+    <mergeCell ref="I6:K7"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="A1:G3"/>
+    <mergeCell ref="H1:N3"/>
+    <mergeCell ref="A4:B5"/>
+    <mergeCell ref="C4:D5"/>
+    <mergeCell ref="E4:H5"/>
+    <mergeCell ref="I4:K5"/>
+    <mergeCell ref="N4:N5"/>
   </mergeCells>
   <conditionalFormatting sqref="B54">
     <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Warning">
@@ -7699,9 +7680,9 @@
       <c r="A2" s="121" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="122" t="str">
+      <c r="B2" s="122">
         <f>'Expense Claim Form '!C4</f>
-        <v>Brian Fleming</v>
+        <v>0</v>
       </c>
       <c r="C2" s="120"/>
       <c r="D2" s="120"/>
@@ -7767,9 +7748,7 @@
       <c r="L4" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="131" t="s">
-        <v>204</v>
-      </c>
+      <c r="M4" s="131"/>
       <c r="N4" s="70"/>
       <c r="O4" s="70"/>
       <c r="P4" s="70"/>
@@ -7794,9 +7773,7 @@
       <c r="L5" s="134" t="s">
         <v>7</v>
       </c>
-      <c r="M5" s="131">
-        <v>1600</v>
-      </c>
+      <c r="M5" s="131"/>
       <c r="N5" s="70"/>
       <c r="O5" s="70"/>
       <c r="P5" s="70"/>
@@ -7828,9 +7805,7 @@
       <c r="L6" s="144" t="s">
         <v>106</v>
       </c>
-      <c r="M6" s="131" t="s">
-        <v>205</v>
-      </c>
+      <c r="M6" s="131"/>
       <c r="N6" s="70"/>
       <c r="O6" s="70"/>
       <c r="P6" s="70"/>
@@ -7862,9 +7837,7 @@
       <c r="L7" s="144" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="131" t="s">
-        <v>206</v>
-      </c>
+      <c r="M7" s="131"/>
       <c r="N7" s="70"/>
       <c r="O7" s="70"/>
       <c r="P7" s="70"/>
@@ -8016,7 +7989,7 @@
       <c r="L12" s="70"/>
       <c r="M12" s="70"/>
       <c r="N12" s="70" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="O12" s="70"/>
       <c r="P12" s="70"/>
@@ -10492,9 +10465,9 @@
       <c r="A2" s="121" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="122" t="str">
+      <c r="B2" s="122">
         <f>'Mileage Detail'!B2</f>
-        <v>Brian Fleming</v>
+        <v>0</v>
       </c>
       <c r="C2" s="120"/>
       <c r="D2" s="120"/>
@@ -10560,9 +10533,7 @@
       <c r="L4" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="131" t="s">
-        <v>204</v>
-      </c>
+      <c r="M4" s="131"/>
       <c r="N4" s="70"/>
       <c r="O4" s="70"/>
       <c r="P4" s="70"/>
@@ -10587,9 +10558,7 @@
       <c r="L5" s="134" t="s">
         <v>7</v>
       </c>
-      <c r="M5" s="131">
-        <v>1600</v>
-      </c>
+      <c r="M5" s="131"/>
       <c r="N5" s="70"/>
       <c r="O5" s="70"/>
       <c r="P5" s="70"/>
@@ -10621,9 +10590,7 @@
       <c r="L6" s="144" t="s">
         <v>106</v>
       </c>
-      <c r="M6" s="131" t="s">
-        <v>205</v>
-      </c>
+      <c r="M6" s="131"/>
       <c r="N6" s="70"/>
       <c r="O6" s="70"/>
       <c r="P6" s="70"/>
@@ -10655,9 +10622,7 @@
       <c r="L7" s="144" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="131" t="s">
-        <v>206</v>
-      </c>
+      <c r="M7" s="131"/>
       <c r="N7" s="70"/>
       <c r="O7" s="70"/>
       <c r="P7" s="70"/>

</xml_diff>